<commit_message>
Add Anderson vs Picard acceleration comparison sweep script
- Implemented a new script `run_anderson_sweep.py` to compare the convergence behavior of Anderson acceleration against Picard iteration across various timesteps.
- Introduced `AndersonSweepConfig` dataclass for configuration management.
- Developed a simulation runner to handle parameter sweeps for different acceleration types and timestep values.
- Configured output structure for results, including CSV and JSON summaries, and visualization data.
- Integrated MPI support for parallel execution.
- Added logging for progress tracking and analysis instructions post-sweep.
</commit_message>
<xml_diff>
--- a/analysis/convergence_analysis/convergence_data.xlsx
+++ b/analysis/convergence_analysis/convergence_data.xlsx
@@ -7,38 +7,41 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="spatial_u_dt6.25" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="spatial_rho_dt6.25" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="spatial_S_dt6.25" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="spatial_A_dt6.25" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="spatial_u_dt12.5" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="spatial_rho_dt12.5" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="spatial_S_dt12.5" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="spatial_A_dt12.5" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="spatial_u_dt25.0" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="spatial_rho_dt25.0" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="spatial_S_dt25.0" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="spatial_A_dt25.0" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="spatial_u_dt50.0" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="spatial_rho_dt50.0" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="spatial_S_dt50.0" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="spatial_A_dt50.0" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="temporal_u_N16" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="temporal_rho_N16" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="temporal_S_N16" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="temporal_A_N16" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="temporal_u_N24" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="temporal_rho_N24" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="temporal_S_N24" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="temporal_A_N24" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="temporal_u_N36" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="temporal_rho_N36" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="temporal_S_N36" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="temporal_A_N36" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="temporal_u_N54" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="temporal_rho_N54" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet name="temporal_S_N54" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet name="temporal_A_N54" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="spatial_psi_dt1.25" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="spatial_rho_dt1.25" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="spatial_S_dt1.25" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="spatial_L_dt1.25" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="spatial_psi_dt2.5" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="spatial_rho_dt2.5" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="spatial_S_dt2.5" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="spatial_L_dt2.5" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="spatial_psi_dt5.0" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="spatial_rho_dt5.0" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="spatial_S_dt5.0" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="spatial_L_dt5.0" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="spatial_psi_dt10.0" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="spatial_rho_dt10.0" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="spatial_S_dt10.0" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="spatial_L_dt10.0" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="spatial_perf_dt1.25" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="spatial_perf_dt2.5" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="spatial_perf_dt5.0" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="spatial_perf_dt10.0" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="temporal_psi_N6" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="temporal_rho_N6" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="temporal_S_N6" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="temporal_L_N6" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="temporal_psi_N12" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="temporal_rho_N12" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="temporal_S_N12" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="temporal_L_N12" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="temporal_psi_N24" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="temporal_rho_N24" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="temporal_S_N24" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="temporal_L_N24" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="temporal_perf_N6" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="temporal_perf_N12" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="temporal_perf_N24" sheetId="35" state="visible" r:id="rId35"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -456,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -483,44 +486,30 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0625</v>
+        <v>1.666666666666667</v>
       </c>
       <c r="C2" t="n">
-        <v>0.00300643393032856</v>
+        <v>0.0002165066251714675</v>
       </c>
       <c r="D2" t="n">
-        <v>0.09565712165626948</v>
+        <v>0.001063196574541369</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B3" t="n">
-        <v>0.04166666666666666</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="C3" t="n">
-        <v>0.001752697762099317</v>
+        <v>0.0001330521554983954</v>
       </c>
       <c r="D3" t="n">
-        <v>0.05820264065180969</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>36</v>
-      </c>
-      <c r="B4" t="n">
-        <v>0.02777777777777778</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.0009039274516627173</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.0333119294232512</v>
+        <v>0.001484327590998175</v>
       </c>
     </row>
   </sheetData>
@@ -534,7 +523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -561,44 +550,30 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0625</v>
+        <v>1.666666666666667</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1110092168902792</v>
+        <v>0.0003530374898045391</v>
       </c>
       <c r="D2" t="n">
-        <v>6.289870335860691</v>
+        <v>6.437879691954515e-05</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B3" t="n">
-        <v>0.04166666666666666</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="C3" t="n">
-        <v>0.07191426995611999</v>
+        <v>0.0001226422445675734</v>
       </c>
       <c r="D3" t="n">
-        <v>4.844285950929366</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>36</v>
-      </c>
-      <c r="B4" t="n">
-        <v>0.02777777777777778</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.0435093498090846</v>
-      </c>
-      <c r="D4" t="n">
-        <v>3.51883470704297</v>
+        <v>4.632816526330397e-05</v>
       </c>
     </row>
   </sheetData>
@@ -612,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -639,44 +614,30 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0625</v>
+        <v>1.666666666666667</v>
       </c>
       <c r="C2" t="n">
-        <v>0.002310022695224693</v>
+        <v>0.001100297050418198</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1410330959516202</v>
+        <v>0.0001709978379974633</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B3" t="n">
-        <v>0.04166666666666666</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="C3" t="n">
-        <v>0.001474584690961879</v>
+        <v>0.0003158082682863014</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1112148031175917</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>36</v>
-      </c>
-      <c r="B4" t="n">
-        <v>0.02777777777777778</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.0008931285531919876</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.08118716726052343</v>
+        <v>8.716570279868264e-05</v>
       </c>
     </row>
   </sheetData>
@@ -690,7 +651,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -717,44 +678,30 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0625</v>
+        <v>1.666666666666667</v>
       </c>
       <c r="C2" t="n">
-        <v>0.01473736156787848</v>
+        <v>0.30250500623027</v>
       </c>
       <c r="D2" t="n">
-        <v>0.127923491483835</v>
+        <v>0.1405328939714831</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B3" t="n">
-        <v>0.04166666666666666</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="C3" t="n">
-        <v>0.00569774788766991</v>
+        <v>0.1536792267675883</v>
       </c>
       <c r="D3" t="n">
-        <v>0.07648628363939559</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>36</v>
-      </c>
-      <c r="B4" t="n">
-        <v>0.02777777777777778</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.003358615577491442</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.04802079790625374</v>
+        <v>0.07697537450433593</v>
       </c>
     </row>
   </sheetData>
@@ -768,7 +715,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -795,44 +742,30 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0625</v>
+        <v>1.666666666666667</v>
       </c>
       <c r="C2" t="n">
-        <v>0.00316029724825373</v>
+        <v>0.0002213412812185539</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1006094546543731</v>
+        <v>0.001084795469978614</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B3" t="n">
-        <v>0.04166666666666666</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="C3" t="n">
-        <v>0.001821363548337093</v>
+        <v>0.000136069167464598</v>
       </c>
       <c r="D3" t="n">
-        <v>0.06026680155688049</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>36</v>
-      </c>
-      <c r="B4" t="n">
-        <v>0.02777777777777778</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.0009630388967660373</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.03441062852310495</v>
+        <v>0.001515768081002552</v>
       </c>
     </row>
   </sheetData>
@@ -846,7 +779,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -873,44 +806,30 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0625</v>
+        <v>1.666666666666667</v>
       </c>
       <c r="C2" t="n">
-        <v>0.117852764328443</v>
+        <v>0.0002555824216906126</v>
       </c>
       <c r="D2" t="n">
-        <v>6.42428571412192</v>
+        <v>6.513716350740936e-05</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B3" t="n">
-        <v>0.04166666666666666</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="C3" t="n">
-        <v>0.07464393363712557</v>
+        <v>7.077774154587844e-05</v>
       </c>
       <c r="D3" t="n">
-        <v>4.923288017521558</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>36</v>
-      </c>
-      <c r="B4" t="n">
-        <v>0.02777777777777778</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.04544650500477405</v>
-      </c>
-      <c r="D4" t="n">
-        <v>3.600043614264182</v>
+        <v>5.597407132422058e-05</v>
       </c>
     </row>
   </sheetData>
@@ -924,7 +843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -951,44 +870,30 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0625</v>
+        <v>1.666666666666667</v>
       </c>
       <c r="C2" t="n">
-        <v>0.002439574202915715</v>
+        <v>0.001132229619195132</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1440671524919648</v>
+        <v>0.0001740569846368793</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B3" t="n">
-        <v>0.04166666666666666</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="C3" t="n">
-        <v>0.001534341509373001</v>
+        <v>0.0003316845664018078</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1136777830983331</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>36</v>
-      </c>
-      <c r="B4" t="n">
-        <v>0.02777777777777778</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.0009299530502887068</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.08322128386124973</v>
+        <v>8.892330683340969e-05</v>
       </c>
     </row>
   </sheetData>
@@ -1002,7 +907,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1029,44 +934,30 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0625</v>
+        <v>1.666666666666667</v>
       </c>
       <c r="C2" t="n">
-        <v>0.01470162345637653</v>
+        <v>0.2990735617555402</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1292092431032767</v>
+        <v>0.1409843443338025</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B3" t="n">
-        <v>0.04166666666666666</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="C3" t="n">
-        <v>0.006074983313566674</v>
+        <v>0.1515259742194704</v>
       </c>
       <c r="D3" t="n">
-        <v>0.07830655513220559</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>36</v>
-      </c>
-      <c r="B4" t="n">
-        <v>0.02777777777777778</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.00336006207325174</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.04854397438487398</v>
+        <v>0.07731280243920619</v>
       </c>
     </row>
   </sheetData>
@@ -1080,57 +971,183 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>dt_days</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>L2_error</t>
-        </is>
-      </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>H1_error</t>
+          <t>mech_iters</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>fab_iters</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>stim_iters</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>dens_iters</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>mech_time</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>fab_time</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>stim_time</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>dens_time</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>memory_mb</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>h</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>6.25</v>
+        <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0004121035980823915</v>
+        <v>1.25</v>
       </c>
       <c r="C2" t="n">
-        <v>0.008943822389025217</v>
+        <v>594</v>
+      </c>
+      <c r="D2" t="n">
+        <v>626</v>
+      </c>
+      <c r="E2" t="n">
+        <v>816</v>
+      </c>
+      <c r="F2" t="n">
+        <v>305</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1.942735901451668</v>
+      </c>
+      <c r="H2" t="n">
+        <v>6.03447765461169</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.2236256413161733</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.4089153861859794</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>1.666666666666667</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>12.5</v>
+        <v>12</v>
       </c>
       <c r="B3" t="n">
-        <v>0.0007065148747088087</v>
+        <v>1.25</v>
       </c>
       <c r="C3" t="n">
-        <v>0.01587850081583747</v>
+        <v>814</v>
+      </c>
+      <c r="D3" t="n">
+        <v>592</v>
+      </c>
+      <c r="E3" t="n">
+        <v>660</v>
+      </c>
+      <c r="F3" t="n">
+        <v>249</v>
+      </c>
+      <c r="G3" t="n">
+        <v>9.828766087768599</v>
+      </c>
+      <c r="H3" t="n">
+        <v>45.03199920151383</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.3055762272560953</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.8499277498340216</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.8333333333333334</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B4" t="n">
-        <v>0.002025659749277964</v>
+        <v>1.25</v>
       </c>
       <c r="C4" t="n">
-        <v>0.05971240947036143</v>
+        <v>1095</v>
+      </c>
+      <c r="D4" t="n">
+        <v>495</v>
+      </c>
+      <c r="E4" t="n">
+        <v>581</v>
+      </c>
+      <c r="F4" t="n">
+        <v>195</v>
+      </c>
+      <c r="G4" t="n">
+        <v>81.95951659360435</v>
+      </c>
+      <c r="H4" t="n">
+        <v>329.6964714269852</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1.516356301843187</v>
+      </c>
+      <c r="J4" t="n">
+        <v>3.331095201661809</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.4166666666666667</v>
       </c>
     </row>
   </sheetData>
@@ -1144,57 +1161,183 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>dt_days</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>L2_error</t>
-        </is>
-      </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>H1_error</t>
+          <t>mech_iters</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>fab_iters</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>stim_iters</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>dens_iters</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>mech_time</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>fab_time</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>stim_time</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>dens_time</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>memory_mb</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>h</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>6.25</v>
+        <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.01862899228874051</v>
+        <v>2.5</v>
       </c>
       <c r="C2" t="n">
-        <v>0.5048915666277943</v>
+        <v>444</v>
+      </c>
+      <c r="D2" t="n">
+        <v>428</v>
+      </c>
+      <c r="E2" t="n">
+        <v>500</v>
+      </c>
+      <c r="F2" t="n">
+        <v>201</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1.201114246039651</v>
+      </c>
+      <c r="H2" t="n">
+        <v>3.518164300243369</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.1097727150190614</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.1727549521019674</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>1.666666666666667</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>12.5</v>
+        <v>12</v>
       </c>
       <c r="B3" t="n">
-        <v>0.03624873593286593</v>
+        <v>2.5</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9857475425023809</v>
+        <v>576</v>
+      </c>
+      <c r="D3" t="n">
+        <v>403</v>
+      </c>
+      <c r="E3" t="n">
+        <v>451</v>
+      </c>
+      <c r="F3" t="n">
+        <v>172</v>
+      </c>
+      <c r="G3" t="n">
+        <v>5.848539495025761</v>
+      </c>
+      <c r="H3" t="n">
+        <v>26.92871816037223</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.2910630808910345</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.5242424521129568</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.8333333333333334</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B4" t="n">
-        <v>0.08900035508259872</v>
+        <v>2.5</v>
       </c>
       <c r="C4" t="n">
-        <v>2.478088632238606</v>
+        <v>739</v>
+      </c>
+      <c r="D4" t="n">
+        <v>363</v>
+      </c>
+      <c r="E4" t="n">
+        <v>444</v>
+      </c>
+      <c r="F4" t="n">
+        <v>126</v>
+      </c>
+      <c r="G4" t="n">
+        <v>50.12723374622874</v>
+      </c>
+      <c r="H4" t="n">
+        <v>199.69873239554</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1.098484682268462</v>
+      </c>
+      <c r="J4" t="n">
+        <v>1.983076842501759</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.4166666666666667</v>
       </c>
     </row>
   </sheetData>
@@ -1208,57 +1351,183 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>dt_days</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>L2_error</t>
-        </is>
-      </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>H1_error</t>
+          <t>mech_iters</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>fab_iters</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>stim_iters</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>dens_iters</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>mech_time</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>fab_time</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>stim_time</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>dens_time</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>memory_mb</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>h</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>6.25</v>
+        <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0003398271510718499</v>
+        <v>5</v>
       </c>
       <c r="C2" t="n">
-        <v>0.009836115767230607</v>
+        <v>305</v>
+      </c>
+      <c r="D2" t="n">
+        <v>284</v>
+      </c>
+      <c r="E2" t="n">
+        <v>299</v>
+      </c>
+      <c r="F2" t="n">
+        <v>145</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.495929772383533</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1.806638952693902</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.0469646060373631</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.0823386751580978</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>1.666666666666667</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>12.5</v>
+        <v>12</v>
       </c>
       <c r="B3" t="n">
-        <v>0.0006511557487703653</v>
+        <v>5</v>
       </c>
       <c r="C3" t="n">
-        <v>0.01884823418618526</v>
+        <v>387</v>
+      </c>
+      <c r="D3" t="n">
+        <v>283</v>
+      </c>
+      <c r="E3" t="n">
+        <v>292</v>
+      </c>
+      <c r="F3" t="n">
+        <v>134</v>
+      </c>
+      <c r="G3" t="n">
+        <v>3.533016937086359</v>
+      </c>
+      <c r="H3" t="n">
+        <v>16.16893683420494</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.1596466174814845</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.3165919564198698</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.8333333333333334</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B4" t="n">
-        <v>0.001595872790276546</v>
+        <v>5</v>
       </c>
       <c r="C4" t="n">
-        <v>0.04722843881626124</v>
+        <v>487</v>
+      </c>
+      <c r="D4" t="n">
+        <v>258</v>
+      </c>
+      <c r="E4" t="n">
+        <v>278</v>
+      </c>
+      <c r="F4" t="n">
+        <v>81</v>
+      </c>
+      <c r="G4" t="n">
+        <v>29.36355632648338</v>
+      </c>
+      <c r="H4" t="n">
+        <v>119.7647395810345</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.5754567530238996</v>
+      </c>
+      <c r="J4" t="n">
+        <v>1.070854557794518</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.4166666666666667</v>
       </c>
     </row>
   </sheetData>
@@ -1272,7 +1541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1299,44 +1568,30 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0625</v>
+        <v>1.666666666666667</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1095809294904612</v>
+        <v>0.0005039764908831473</v>
       </c>
       <c r="D2" t="n">
-        <v>6.267272885611727</v>
+        <v>4.017255439622285e-05</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B3" t="n">
-        <v>0.04166666666666666</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="C3" t="n">
-        <v>0.07150310603156106</v>
+        <v>0.0006362737802515334</v>
       </c>
       <c r="D3" t="n">
-        <v>4.857154946861646</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>36</v>
-      </c>
-      <c r="B4" t="n">
-        <v>0.02777777777777778</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.04276366463918945</v>
-      </c>
-      <c r="D4" t="n">
-        <v>3.512601650964549</v>
+        <v>3.208310685395392e-05</v>
       </c>
     </row>
   </sheetData>
@@ -1350,57 +1605,183 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>dt_days</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>L2_error</t>
-        </is>
-      </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>H1_error</t>
+          <t>mech_iters</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>fab_iters</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>stim_iters</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>dens_iters</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>mech_time</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>fab_time</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>stim_time</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>dens_time</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>memory_mb</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>h</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>6.25</v>
+        <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.00135180534764553</v>
+        <v>10</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0105518424632717</v>
+        <v>201</v>
+      </c>
+      <c r="D2" t="n">
+        <v>200</v>
+      </c>
+      <c r="E2" t="n">
+        <v>185</v>
+      </c>
+      <c r="F2" t="n">
+        <v>108</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.2600158952409399</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.9956688375677911</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.0221955819288266</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.0434778656344858</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>1.666666666666667</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>12.5</v>
+        <v>12</v>
       </c>
       <c r="B3" t="n">
-        <v>0.002229674611459152</v>
+        <v>10</v>
       </c>
       <c r="C3" t="n">
-        <v>0.01734916395928449</v>
+        <v>252</v>
+      </c>
+      <c r="D3" t="n">
+        <v>208</v>
+      </c>
+      <c r="E3" t="n">
+        <v>185</v>
+      </c>
+      <c r="F3" t="n">
+        <v>79</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2.15053381875623</v>
+      </c>
+      <c r="H3" t="n">
+        <v>10.16239234420937</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.1018874311121179</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.1465309080667791</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.8333333333333334</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B4" t="n">
-        <v>0.00552716965592462</v>
+        <v>10</v>
       </c>
       <c r="C4" t="n">
-        <v>0.04830219261379191</v>
+        <v>316</v>
+      </c>
+      <c r="D4" t="n">
+        <v>189</v>
+      </c>
+      <c r="E4" t="n">
+        <v>172</v>
+      </c>
+      <c r="F4" t="n">
+        <v>64</v>
+      </c>
+      <c r="G4" t="n">
+        <v>16.84581571863964</v>
+      </c>
+      <c r="H4" t="n">
+        <v>69.68289785645902</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.3953183108242226</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.6184828691184521</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.4166666666666667</v>
       </c>
     </row>
   </sheetData>
@@ -1436,35 +1817,35 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>6.25</v>
+        <v>10</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0003357302723511506</v>
+        <v>2.283952020104065e-05</v>
       </c>
       <c r="C2" t="n">
-        <v>0.005976794281624305</v>
+        <v>6.485817999376512e-06</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>12.5</v>
+        <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.0006341501060855648</v>
+        <v>1.23490213969495e-05</v>
       </c>
       <c r="C3" t="n">
-        <v>0.01170331656074314</v>
+        <v>3.538613945712992e-06</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>25</v>
+        <v>2.5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.001458419770223554</v>
+        <v>6.383905579461187e-06</v>
       </c>
       <c r="C4" t="n">
-        <v>0.03147921665869582</v>
+        <v>1.835764503536061e-06</v>
       </c>
     </row>
   </sheetData>
@@ -1500,35 +1881,35 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>6.25</v>
+        <v>10</v>
       </c>
       <c r="B2" t="n">
-        <v>0.01961348723446566</v>
+        <v>0.006075574639456593</v>
       </c>
       <c r="C2" t="n">
-        <v>0.5636511968946342</v>
+        <v>1.073194520666682e-05</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>12.5</v>
+        <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.03784154723324491</v>
+        <v>0.0004564455520853383</v>
       </c>
       <c r="C3" t="n">
-        <v>1.091223618503808</v>
+        <v>1.145256687848298e-05</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>25</v>
+        <v>2.5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.09427542021603603</v>
+        <v>0.0008570885772742201</v>
       </c>
       <c r="C4" t="n">
-        <v>2.756853929494582</v>
+        <v>4.451639001809863e-06</v>
       </c>
     </row>
   </sheetData>
@@ -1564,35 +1945,35 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>6.25</v>
+        <v>10</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0003667563381902967</v>
+        <v>1.053766619249608</v>
       </c>
       <c r="C2" t="n">
-        <v>0.01116722719453216</v>
+        <v>7.826158373435056e-06</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>12.5</v>
+        <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.0006995124892050047</v>
+        <v>0.5548410337136515</v>
       </c>
       <c r="C3" t="n">
-        <v>0.02155982268440002</v>
+        <v>4.502569880365119e-06</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>25</v>
+        <v>2.5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.001728177430535912</v>
+        <v>0.2846303126112653</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0542742185196907</v>
+        <v>2.410363658642893e-06</v>
       </c>
     </row>
   </sheetData>
@@ -1628,35 +2009,35 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>6.25</v>
+        <v>10</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0009556082348092218</v>
+        <v>0.8234139584034206</v>
       </c>
       <c r="C2" t="n">
-        <v>0.008552265075650626</v>
+        <v>0.005020005879844958</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>12.5</v>
+        <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.001761927486952603</v>
+        <v>0.4362134940104586</v>
       </c>
       <c r="C3" t="n">
-        <v>0.01680117637253449</v>
+        <v>0.002443447207783183</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>25</v>
+        <v>2.5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.003826438891211597</v>
+        <v>0.2247498716914258</v>
       </c>
       <c r="C4" t="n">
-        <v>0.03873875914351586</v>
+        <v>0.001217740722571841</v>
       </c>
     </row>
   </sheetData>
@@ -1692,35 +2073,35 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>6.25</v>
+        <v>10</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0002954903002005387</v>
+        <v>2.435090788182105e-05</v>
       </c>
       <c r="C2" t="n">
-        <v>0.003827227537707811</v>
+        <v>9.966834606614709e-06</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>12.5</v>
+        <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.0005594326045206667</v>
+        <v>1.31675255232795e-05</v>
       </c>
       <c r="C3" t="n">
-        <v>0.007820417853119993</v>
+        <v>5.425767932543056e-06</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>25</v>
+        <v>2.5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.001399291613503711</v>
+        <v>6.80119844390595e-06</v>
       </c>
       <c r="C4" t="n">
-        <v>0.02172075307761157</v>
+        <v>2.810309027759479e-06</v>
       </c>
     </row>
   </sheetData>
@@ -1756,35 +2137,35 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>6.25</v>
+        <v>10</v>
       </c>
       <c r="B2" t="n">
-        <v>0.01762345936914248</v>
+        <v>0.005975346363929602</v>
       </c>
       <c r="C2" t="n">
-        <v>0.5206848947389309</v>
+        <v>1.6761527996245e-05</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>12.5</v>
+        <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.03524996691369112</v>
+        <v>0.0005471677457735829</v>
       </c>
       <c r="C3" t="n">
-        <v>1.050257821521306</v>
+        <v>5.363915806981764e-05</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>25</v>
+        <v>2.5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.09968346025630294</v>
+        <v>0.000919632769937976</v>
       </c>
       <c r="C4" t="n">
-        <v>3.002257536524471</v>
+        <v>1.004568104922954e-05</v>
       </c>
     </row>
   </sheetData>
@@ -1820,35 +2201,35 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>6.25</v>
+        <v>10</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0003394859227755243</v>
+        <v>1.053798173027476</v>
       </c>
       <c r="C2" t="n">
-        <v>0.01040352441474933</v>
+        <v>9.64896707041137e-06</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>12.5</v>
+        <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.0006680569740977374</v>
+        <v>0.5548590073188699</v>
       </c>
       <c r="C3" t="n">
-        <v>0.02081310921772093</v>
+        <v>5.724290790597855e-06</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>25</v>
+        <v>2.5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.001842794178616721</v>
+        <v>0.2846399774156555</v>
       </c>
       <c r="C4" t="n">
-        <v>0.05910355117016863</v>
+        <v>3.299019339369593e-06</v>
       </c>
     </row>
   </sheetData>
@@ -1884,35 +2265,35 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>6.25</v>
+        <v>10</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0007980613766841364</v>
+        <v>0.825360866933887</v>
       </c>
       <c r="C2" t="n">
-        <v>0.007255919178275058</v>
+        <v>0.005423768636990894</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>12.5</v>
+        <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.001431861552630523</v>
+        <v>0.4373252135051868</v>
       </c>
       <c r="C3" t="n">
-        <v>0.01447928913534449</v>
+        <v>0.002647555287699452</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>25</v>
+        <v>2.5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.003485269956050854</v>
+        <v>0.2251513354646406</v>
       </c>
       <c r="C4" t="n">
-        <v>0.03826135663651827</v>
+        <v>0.001315904992786004</v>
       </c>
     </row>
   </sheetData>
@@ -1948,35 +2329,35 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>6.25</v>
+        <v>10</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0002700013265751651</v>
+        <v>2.487479579809256e-05</v>
       </c>
       <c r="C2" t="n">
-        <v>0.003434469801571375</v>
+        <v>1.336892027332579e-05</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>12.5</v>
+        <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.000516385600780985</v>
+        <v>1.347918204492729e-05</v>
       </c>
       <c r="C3" t="n">
-        <v>0.006987693190946321</v>
+        <v>7.295815298528894e-06</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>25</v>
+        <v>2.5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.00138870328503209</v>
+        <v>6.973496948096739e-06</v>
       </c>
       <c r="C4" t="n">
-        <v>0.02112167489775546</v>
+        <v>3.785819558686972e-06</v>
       </c>
     </row>
   </sheetData>
@@ -1990,7 +2371,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2017,44 +2398,30 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0625</v>
+        <v>1.666666666666667</v>
       </c>
       <c r="C2" t="n">
-        <v>0.002281281076236551</v>
+        <v>0.001072129878348777</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1410301793270706</v>
+        <v>0.0001678843819080905</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B3" t="n">
-        <v>0.04166666666666666</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="C3" t="n">
-        <v>0.001457957772101036</v>
+        <v>0.0003066067181270852</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1109604098236228</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>36</v>
-      </c>
-      <c r="B4" t="n">
-        <v>0.02777777777777778</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.0008751898167828485</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.08098188563057007</v>
+        <v>8.551156136940436e-05</v>
       </c>
     </row>
   </sheetData>
@@ -2090,35 +2457,35 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>6.25</v>
+        <v>10</v>
       </c>
       <c r="B2" t="n">
-        <v>0.01688911073034806</v>
+        <v>0.005792642922764942</v>
       </c>
       <c r="C2" t="n">
-        <v>0.5125085961229079</v>
+        <v>3.672918421320289e-05</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>12.5</v>
+        <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.03376991370670529</v>
+        <v>0.000960584664871514</v>
       </c>
       <c r="C3" t="n">
-        <v>1.031898660665288</v>
+        <v>4.769419484334612e-06</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>25</v>
+        <v>2.5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.1014608622105396</v>
+        <v>0.001022288856160226</v>
       </c>
       <c r="C4" t="n">
-        <v>3.106123323945603</v>
+        <v>1.696535846296647e-05</v>
       </c>
     </row>
   </sheetData>
@@ -2154,35 +2521,35 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>6.25</v>
+        <v>10</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0003294911015464927</v>
+        <v>1.053813789316715</v>
       </c>
       <c r="C2" t="n">
-        <v>0.01028683910611494</v>
+        <v>1.083703786542882e-05</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>12.5</v>
+        <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.0006481545781063268</v>
+        <v>0.5548638227990698</v>
       </c>
       <c r="C3" t="n">
-        <v>0.02052500579288228</v>
+        <v>7.076079904009496e-06</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>25</v>
+        <v>2.5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.001882673055339634</v>
+        <v>0.28464383677072</v>
       </c>
       <c r="C4" t="n">
-        <v>0.06110681388200048</v>
+        <v>1.028569216643447e-05</v>
       </c>
     </row>
   </sheetData>
@@ -2218,35 +2585,668 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>6.25</v>
+        <v>10</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0007363312285211183</v>
+        <v>0.8268445285239455</v>
       </c>
       <c r="C2" t="n">
-        <v>0.006699535157313847</v>
+        <v>0.005779182692318237</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>12.5</v>
+        <v>5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.001310959658048085</v>
+        <v>0.4382024391807939</v>
       </c>
       <c r="C3" t="n">
-        <v>0.01336260175997275</v>
+        <v>0.002834669009020767</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>25</v>
+        <v>2.5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.003413582511922756</v>
+        <v>0.226202058276449</v>
       </c>
       <c r="C4" t="n">
-        <v>0.03832710291845508</v>
+        <v>0.001408613242416547</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>dt_days</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>mech_iters</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>fab_iters</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>stim_iters</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>dens_iters</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>mech_time</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>fab_time</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>stim_time</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>dens_time</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>memory_mb</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C2" t="n">
+        <v>201</v>
+      </c>
+      <c r="D2" t="n">
+        <v>200</v>
+      </c>
+      <c r="E2" t="n">
+        <v>185</v>
+      </c>
+      <c r="F2" t="n">
+        <v>108</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.2600158952409399</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.9956688375677911</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.0221955819288266</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.0434778656344858</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3" t="n">
+        <v>305</v>
+      </c>
+      <c r="D3" t="n">
+        <v>284</v>
+      </c>
+      <c r="E3" t="n">
+        <v>299</v>
+      </c>
+      <c r="F3" t="n">
+        <v>145</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.495929772383533</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1.806638952693902</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.0469646060373631</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.0823386751580978</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C4" t="n">
+        <v>444</v>
+      </c>
+      <c r="D4" t="n">
+        <v>428</v>
+      </c>
+      <c r="E4" t="n">
+        <v>500</v>
+      </c>
+      <c r="F4" t="n">
+        <v>201</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1.201114246039651</v>
+      </c>
+      <c r="H4" t="n">
+        <v>3.518164300243369</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.1097727150190614</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.1727549521019674</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B5" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="C5" t="n">
+        <v>594</v>
+      </c>
+      <c r="D5" t="n">
+        <v>626</v>
+      </c>
+      <c r="E5" t="n">
+        <v>816</v>
+      </c>
+      <c r="F5" t="n">
+        <v>305</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1.942735901451668</v>
+      </c>
+      <c r="H5" t="n">
+        <v>6.03447765461169</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.2236256413161733</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.4089153861859794</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>dt_days</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>mech_iters</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>fab_iters</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>stim_iters</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>dens_iters</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>mech_time</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>fab_time</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>stim_time</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>dens_time</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>memory_mb</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C2" t="n">
+        <v>252</v>
+      </c>
+      <c r="D2" t="n">
+        <v>208</v>
+      </c>
+      <c r="E2" t="n">
+        <v>185</v>
+      </c>
+      <c r="F2" t="n">
+        <v>79</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2.15053381875623</v>
+      </c>
+      <c r="H2" t="n">
+        <v>10.16239234420937</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.1018874311121179</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.1465309080667791</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3" t="n">
+        <v>387</v>
+      </c>
+      <c r="D3" t="n">
+        <v>283</v>
+      </c>
+      <c r="E3" t="n">
+        <v>292</v>
+      </c>
+      <c r="F3" t="n">
+        <v>134</v>
+      </c>
+      <c r="G3" t="n">
+        <v>3.533016937086359</v>
+      </c>
+      <c r="H3" t="n">
+        <v>16.16893683420494</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.1596466174814845</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.3165919564198698</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C4" t="n">
+        <v>576</v>
+      </c>
+      <c r="D4" t="n">
+        <v>403</v>
+      </c>
+      <c r="E4" t="n">
+        <v>451</v>
+      </c>
+      <c r="F4" t="n">
+        <v>172</v>
+      </c>
+      <c r="G4" t="n">
+        <v>5.848539495025761</v>
+      </c>
+      <c r="H4" t="n">
+        <v>26.92871816037223</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.2910630808910345</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.5242424521129568</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B5" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="C5" t="n">
+        <v>814</v>
+      </c>
+      <c r="D5" t="n">
+        <v>592</v>
+      </c>
+      <c r="E5" t="n">
+        <v>660</v>
+      </c>
+      <c r="F5" t="n">
+        <v>249</v>
+      </c>
+      <c r="G5" t="n">
+        <v>9.828766087768599</v>
+      </c>
+      <c r="H5" t="n">
+        <v>45.03199920151383</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.3055762272560953</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.8499277498340216</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>dt_days</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>mech_iters</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>fab_iters</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>stim_iters</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>dens_iters</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>mech_time</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>fab_time</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>stim_time</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>dens_time</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>memory_mb</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C2" t="n">
+        <v>316</v>
+      </c>
+      <c r="D2" t="n">
+        <v>189</v>
+      </c>
+      <c r="E2" t="n">
+        <v>172</v>
+      </c>
+      <c r="F2" t="n">
+        <v>64</v>
+      </c>
+      <c r="G2" t="n">
+        <v>16.84581571863964</v>
+      </c>
+      <c r="H2" t="n">
+        <v>69.68289785645902</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.3953183108242226</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.6184828691184521</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3" t="n">
+        <v>487</v>
+      </c>
+      <c r="D3" t="n">
+        <v>258</v>
+      </c>
+      <c r="E3" t="n">
+        <v>278</v>
+      </c>
+      <c r="F3" t="n">
+        <v>81</v>
+      </c>
+      <c r="G3" t="n">
+        <v>29.36355632648338</v>
+      </c>
+      <c r="H3" t="n">
+        <v>119.7647395810345</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.5754567530238996</v>
+      </c>
+      <c r="J3" t="n">
+        <v>1.070854557794518</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>24</v>
+      </c>
+      <c r="B4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C4" t="n">
+        <v>739</v>
+      </c>
+      <c r="D4" t="n">
+        <v>363</v>
+      </c>
+      <c r="E4" t="n">
+        <v>444</v>
+      </c>
+      <c r="F4" t="n">
+        <v>126</v>
+      </c>
+      <c r="G4" t="n">
+        <v>50.12723374622874</v>
+      </c>
+      <c r="H4" t="n">
+        <v>199.69873239554</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1.098484682268462</v>
+      </c>
+      <c r="J4" t="n">
+        <v>1.983076842501759</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>24</v>
+      </c>
+      <c r="B5" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1095</v>
+      </c>
+      <c r="D5" t="n">
+        <v>495</v>
+      </c>
+      <c r="E5" t="n">
+        <v>581</v>
+      </c>
+      <c r="F5" t="n">
+        <v>195</v>
+      </c>
+      <c r="G5" t="n">
+        <v>81.95951659360435</v>
+      </c>
+      <c r="H5" t="n">
+        <v>329.6964714269852</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1.516356301843187</v>
+      </c>
+      <c r="J5" t="n">
+        <v>3.331095201661809</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2260,7 +3260,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2287,44 +3287,30 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0625</v>
+        <v>1.666666666666667</v>
       </c>
       <c r="C2" t="n">
-        <v>0.01379622230297744</v>
+        <v>0.3048230107027982</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1257399165384232</v>
+        <v>0.1399865301816465</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B3" t="n">
-        <v>0.04166666666666666</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="C3" t="n">
-        <v>0.005611464446161946</v>
+        <v>0.1553716538728812</v>
       </c>
       <c r="D3" t="n">
-        <v>0.07651853006675904</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>36</v>
-      </c>
-      <c r="B4" t="n">
-        <v>0.02777777777777778</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.003442461863118394</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.04801752513292946</v>
+        <v>0.07661105779335059</v>
       </c>
     </row>
   </sheetData>
@@ -2338,7 +3324,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2365,44 +3351,30 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0625</v>
+        <v>1.666666666666667</v>
       </c>
       <c r="C2" t="n">
-        <v>0.003064992681160395</v>
+        <v>0.000217251907391458</v>
       </c>
       <c r="D2" t="n">
-        <v>0.09567116585151553</v>
+        <v>0.001066551400352979</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B3" t="n">
-        <v>0.04166666666666666</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="C3" t="n">
-        <v>0.001761602519111352</v>
+        <v>0.0001335232147441913</v>
       </c>
       <c r="D3" t="n">
-        <v>0.05831176078129709</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>36</v>
-      </c>
-      <c r="B4" t="n">
-        <v>0.02777777777777778</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.000917783638904381</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.03327668674224997</v>
+        <v>0.001489209484166055</v>
       </c>
     </row>
   </sheetData>
@@ -2416,7 +3388,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2443,44 +3415,30 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0625</v>
+        <v>1.666666666666667</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1096910872118942</v>
+        <v>0.0004419837641315517</v>
       </c>
       <c r="D2" t="n">
-        <v>6.2666834971464</v>
+        <v>4.170505714143223e-05</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B3" t="n">
-        <v>0.04166666666666666</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="C3" t="n">
-        <v>0.07155068325595253</v>
+        <v>0.0005337530224208233</v>
       </c>
       <c r="D3" t="n">
-        <v>4.848447585862108</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>36</v>
-      </c>
-      <c r="B4" t="n">
-        <v>0.02777777777777778</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.04301736331180706</v>
-      </c>
-      <c r="D4" t="n">
-        <v>3.511736649340386</v>
+        <v>2.752645411890347e-05</v>
       </c>
     </row>
   </sheetData>
@@ -2494,7 +3452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2521,44 +3479,30 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0625</v>
+        <v>1.666666666666667</v>
       </c>
       <c r="C2" t="n">
-        <v>0.002283717387244401</v>
+        <v>0.001082040226802994</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1408322983914072</v>
+        <v>0.0001690796112215444</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B3" t="n">
-        <v>0.04166666666666666</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="C3" t="n">
-        <v>0.001461982499677674</v>
+        <v>0.0003107385955981887</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1109440270023699</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>36</v>
-      </c>
-      <c r="B4" t="n">
-        <v>0.02777777777777778</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.0008809589448608102</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.0809824389677391</v>
+        <v>8.648906227753302e-05</v>
       </c>
     </row>
   </sheetData>
@@ -2572,7 +3516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2599,44 +3543,30 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0625</v>
+        <v>1.666666666666667</v>
       </c>
       <c r="C2" t="n">
-        <v>0.01417481007587593</v>
+        <v>0.3040927853529095</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1265568886748156</v>
+        <v>0.1401877307418837</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B3" t="n">
-        <v>0.04166666666666666</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="C3" t="n">
-        <v>0.00562008375454225</v>
+        <v>0.154734169453263</v>
       </c>
       <c r="D3" t="n">
-        <v>0.07649377604415569</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>36</v>
-      </c>
-      <c r="B4" t="n">
-        <v>0.02777777777777778</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.003409448196959942</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.04800824287381136</v>
+        <v>0.07674175209813321</v>
       </c>
     </row>
   </sheetData>
@@ -2650,7 +3580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2677,44 +3607,30 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0625</v>
+        <v>1.666666666666667</v>
       </c>
       <c r="C2" t="n">
-        <v>0.003162955205037106</v>
+        <v>0.0002186950518489271</v>
       </c>
       <c r="D2" t="n">
-        <v>0.09627503736283979</v>
+        <v>0.00107301218558512</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B3" t="n">
-        <v>0.04166666666666666</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="C3" t="n">
-        <v>0.001773201052272029</v>
+        <v>0.0001344267620392627</v>
       </c>
       <c r="D3" t="n">
-        <v>0.05849290821275318</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>36</v>
-      </c>
-      <c r="B4" t="n">
-        <v>0.02777777777777778</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0.0009368213792342752</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.03332480062303642</v>
+        <v>0.001498612008468028</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor anderson diagnostic plotting: update colorbar positioning, adjust legend locations, and modify output file naming
</commit_message>
<xml_diff>
--- a/analysis/convergence_analysis/convergence_data.xlsx
+++ b/analysis/convergence_analysis/convergence_data.xlsx
@@ -502,10 +502,10 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0002460218585670572</v>
+        <v>0.0002005051526942156</v>
       </c>
       <c r="D2" t="n">
-        <v>0.002186543895629811</v>
+        <v>0.001896873028870768</v>
       </c>
     </row>
     <row r="3">
@@ -516,10 +516,10 @@
         <v>0.625</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0002200910987149827</v>
+        <v>0.0001931055839136455</v>
       </c>
       <c r="D3" t="n">
-        <v>0.00293874080061283</v>
+        <v>0.002611596771114187</v>
       </c>
     </row>
     <row r="4">
@@ -530,10 +530,10 @@
         <v>0.4166666666666667</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0001512167611147858</v>
+        <v>0.0001378823949247219</v>
       </c>
       <c r="D4" t="n">
-        <v>0.002914847823939986</v>
+        <v>0.002684404104403442</v>
       </c>
     </row>
   </sheetData>
@@ -580,10 +580,10 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="C2" t="n">
-        <v>0.94716238138959</v>
+        <v>0.1699483172156054</v>
       </c>
       <c r="D2" t="n">
-        <v>4.643017430792033</v>
+        <v>0.5249423959644979</v>
       </c>
     </row>
     <row r="3">
@@ -594,10 +594,10 @@
         <v>0.625</v>
       </c>
       <c r="C3" t="n">
-        <v>0.6850772054281264</v>
+        <v>0.1238443828834275</v>
       </c>
       <c r="D3" t="n">
-        <v>3.238060613720304</v>
+        <v>0.4162045251904196</v>
       </c>
     </row>
     <row r="4">
@@ -608,10 +608,10 @@
         <v>0.4166666666666667</v>
       </c>
       <c r="C4" t="n">
-        <v>0.2974653524308851</v>
+        <v>0.04992027169161291</v>
       </c>
       <c r="D4" t="n">
-        <v>2.883462319605233</v>
+        <v>0.3742951759743514</v>
       </c>
     </row>
   </sheetData>
@@ -658,10 +658,10 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="C2" t="n">
-        <v>0.3959152904273315</v>
+        <v>0.9099951350291752</v>
       </c>
       <c r="D2" t="n">
-        <v>1.537687173636545</v>
+        <v>3.359909405818444</v>
       </c>
     </row>
     <row r="3">
@@ -672,10 +672,10 @@
         <v>0.625</v>
       </c>
       <c r="C3" t="n">
-        <v>0.2790370004892646</v>
+        <v>0.6979078037810602</v>
       </c>
       <c r="D3" t="n">
-        <v>1.120153916488621</v>
+        <v>2.814369845817308</v>
       </c>
     </row>
     <row r="4">
@@ -686,10 +686,10 @@
         <v>0.4166666666666667</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1181466917942204</v>
+        <v>0.3011388688497764</v>
       </c>
       <c r="D4" t="n">
-        <v>1.008496151908853</v>
+        <v>2.55319342361532</v>
       </c>
     </row>
   </sheetData>
@@ -736,10 +736,10 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="C2" t="n">
-        <v>0.3273582364589959</v>
+        <v>0.3047971956943637</v>
       </c>
       <c r="D2" t="n">
-        <v>1.020269325065878</v>
+        <v>0.824506976059071</v>
       </c>
     </row>
     <row r="3">
@@ -750,10 +750,10 @@
         <v>0.625</v>
       </c>
       <c r="C3" t="n">
-        <v>0.2973967949762574</v>
+        <v>0.2701872310550197</v>
       </c>
       <c r="D3" t="n">
-        <v>0.7293654865028436</v>
+        <v>0.6245345764452926</v>
       </c>
     </row>
     <row r="4">
@@ -764,10 +764,10 @@
         <v>0.4166666666666667</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1338916736913656</v>
+        <v>0.1180630909765896</v>
       </c>
       <c r="D4" t="n">
-        <v>0.63577726057637</v>
+        <v>0.5388026274244215</v>
       </c>
     </row>
   </sheetData>
@@ -814,10 +814,10 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0002233908278308683</v>
+        <v>0.0002017213409160031</v>
       </c>
       <c r="D2" t="n">
-        <v>0.001946327793644166</v>
+        <v>0.001908721937173041</v>
       </c>
     </row>
     <row r="3">
@@ -828,10 +828,10 @@
         <v>0.625</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0001964166135412329</v>
+        <v>0.0001948844793252612</v>
       </c>
       <c r="D3" t="n">
-        <v>0.00262192860930284</v>
+        <v>0.002635055027754604</v>
       </c>
     </row>
     <row r="4">
@@ -842,10 +842,10 @@
         <v>0.4166666666666667</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0001364585492769597</v>
+        <v>0.0001391982478841734</v>
       </c>
       <c r="D4" t="n">
-        <v>0.002635523770578931</v>
+        <v>0.002710786243809959</v>
       </c>
     </row>
   </sheetData>
@@ -892,10 +892,10 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9599058047338609</v>
+        <v>0.1654603294609069</v>
       </c>
       <c r="D2" t="n">
-        <v>4.538149743560542</v>
+        <v>0.5104153623809737</v>
       </c>
     </row>
     <row r="3">
@@ -906,10 +906,10 @@
         <v>0.625</v>
       </c>
       <c r="C3" t="n">
-        <v>0.6673214024444466</v>
+        <v>0.1190952102142002</v>
       </c>
       <c r="D3" t="n">
-        <v>3.170817392680333</v>
+        <v>0.4057146062794245</v>
       </c>
     </row>
     <row r="4">
@@ -920,10 +920,10 @@
         <v>0.4166666666666667</v>
       </c>
       <c r="C4" t="n">
-        <v>0.2869648447746196</v>
+        <v>0.04812015159889488</v>
       </c>
       <c r="D4" t="n">
-        <v>2.834644776046714</v>
+        <v>0.365032172190292</v>
       </c>
     </row>
   </sheetData>
@@ -970,10 +970,10 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="C2" t="n">
-        <v>0.4177954104534496</v>
+        <v>0.8759544822557336</v>
       </c>
       <c r="D2" t="n">
-        <v>1.55779614152393</v>
+        <v>3.283088132169308</v>
       </c>
     </row>
     <row r="3">
@@ -984,10 +984,10 @@
         <v>0.625</v>
       </c>
       <c r="C3" t="n">
-        <v>0.2902909387158927</v>
+        <v>0.6792360920671902</v>
       </c>
       <c r="D3" t="n">
-        <v>1.131010602622142</v>
+        <v>2.76171806062233</v>
       </c>
     </row>
     <row r="4">
@@ -998,10 +998,10 @@
         <v>0.4166666666666667</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1218457214496236</v>
+        <v>0.2926431835548112</v>
       </c>
       <c r="D4" t="n">
-        <v>1.022097504315499</v>
+        <v>2.50177438520653</v>
       </c>
     </row>
   </sheetData>
@@ -1048,10 +1048,10 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="C2" t="n">
-        <v>0.3283905904978489</v>
+        <v>0.2921678294465208</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9983984830195375</v>
+        <v>0.7946938468411832</v>
       </c>
     </row>
     <row r="3">
@@ -1062,10 +1062,10 @@
         <v>0.625</v>
       </c>
       <c r="C3" t="n">
-        <v>0.2977159047650129</v>
+        <v>0.2591473238611288</v>
       </c>
       <c r="D3" t="n">
-        <v>0.7141775150157345</v>
+        <v>0.6017496381216678</v>
       </c>
     </row>
     <row r="4">
@@ -1076,10 +1076,10 @@
         <v>0.4166666666666667</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1333437665219969</v>
+        <v>0.113298112603027</v>
       </c>
       <c r="D4" t="n">
-        <v>0.6223801001964745</v>
+        <v>0.5193817503269411</v>
       </c>
     </row>
   </sheetData>
@@ -1126,10 +1126,10 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0002143789059733602</v>
+        <v>0.0002031508170078398</v>
       </c>
       <c r="D2" t="n">
-        <v>0.00180967895120951</v>
+        <v>0.001922505137325009</v>
       </c>
     </row>
     <row r="3">
@@ -1140,10 +1140,10 @@
         <v>0.625</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0001905292135578782</v>
+        <v>0.0001968565507961578</v>
       </c>
       <c r="D3" t="n">
-        <v>0.002497877592791713</v>
+        <v>0.002661114816777545</v>
       </c>
     </row>
     <row r="4">
@@ -1154,10 +1154,10 @@
         <v>0.4166666666666667</v>
       </c>
       <c r="C4" t="n">
-        <v>0.000131660297374458</v>
+        <v>0.0001406494744762329</v>
       </c>
       <c r="D4" t="n">
-        <v>0.002525510844667061</v>
+        <v>0.002739805078022601</v>
       </c>
     </row>
   </sheetData>
@@ -1204,10 +1204,10 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="C2" t="n">
-        <v>1.17765670125166</v>
+        <v>0.1587811324294244</v>
       </c>
       <c r="D2" t="n">
-        <v>4.19079170885704</v>
+        <v>0.4876973264325958</v>
       </c>
     </row>
     <row r="3">
@@ -1218,10 +1218,10 @@
         <v>0.625</v>
       </c>
       <c r="C3" t="n">
-        <v>0.7558954590570175</v>
+        <v>0.1115874802194794</v>
       </c>
       <c r="D3" t="n">
-        <v>2.904407868562533</v>
+        <v>0.3883366546659042</v>
       </c>
     </row>
     <row r="4">
@@ -1232,10 +1232,10 @@
         <v>0.4166666666666667</v>
       </c>
       <c r="C4" t="n">
-        <v>0.3039030171575382</v>
+        <v>0.04514731455203786</v>
       </c>
       <c r="D4" t="n">
-        <v>2.613488639464504</v>
+        <v>0.3494825750304648</v>
       </c>
     </row>
   </sheetData>
@@ -1282,10 +1282,10 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="C2" t="n">
-        <v>0.4973546519686192</v>
+        <v>0.8273015551242165</v>
       </c>
       <c r="D2" t="n">
-        <v>1.578690644687966</v>
+        <v>3.193525771386882</v>
       </c>
     </row>
     <row r="3">
@@ -1296,10 +1296,10 @@
         <v>0.625</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3379823599909177</v>
+        <v>0.6511477844876156</v>
       </c>
       <c r="D3" t="n">
-        <v>1.145453771038176</v>
+        <v>2.691544850893608</v>
       </c>
     </row>
     <row r="4">
@@ -1310,10 +1310,10 @@
         <v>0.4166666666666667</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1389189411112741</v>
+        <v>0.2798516939220767</v>
       </c>
       <c r="D4" t="n">
-        <v>1.03586922847202</v>
+        <v>2.432847845206855</v>
       </c>
     </row>
   </sheetData>
@@ -1360,10 +1360,10 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9210671891181696</v>
+        <v>0.1739208242585174</v>
       </c>
       <c r="D2" t="n">
-        <v>4.628549515713707</v>
+        <v>0.5377671484874261</v>
       </c>
     </row>
     <row r="3">
@@ -1374,10 +1374,10 @@
         <v>0.625</v>
       </c>
       <c r="C3" t="n">
-        <v>0.6676861939852082</v>
+        <v>0.1279271833814142</v>
       </c>
       <c r="D3" t="n">
-        <v>3.21194333086057</v>
+        <v>0.4251912858253198</v>
       </c>
     </row>
     <row r="4">
@@ -1388,10 +1388,10 @@
         <v>0.4166666666666667</v>
       </c>
       <c r="C4" t="n">
-        <v>0.2907983935021538</v>
+        <v>0.05143377664413997</v>
       </c>
       <c r="D4" t="n">
-        <v>2.860016995199799</v>
+        <v>0.3821418072804961</v>
       </c>
     </row>
   </sheetData>
@@ -1438,10 +1438,10 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="C2" t="n">
-        <v>0.3460121969849416</v>
+        <v>0.2694485927904814</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9724613465144643</v>
+        <v>0.7415897889563989</v>
       </c>
     </row>
     <row r="3">
@@ -1452,10 +1452,10 @@
         <v>0.625</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3080750459017937</v>
+        <v>0.2396562324082627</v>
       </c>
       <c r="D3" t="n">
-        <v>0.6973259870605145</v>
+        <v>0.5610498733196612</v>
       </c>
     </row>
     <row r="4">
@@ -1466,10 +1466,10 @@
         <v>0.4166666666666667</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1356274371110693</v>
+        <v>0.1050150049603432</v>
       </c>
       <c r="D4" t="n">
-        <v>0.6059699152838758</v>
+        <v>0.4846659411735125</v>
       </c>
     </row>
   </sheetData>
@@ -1556,31 +1556,31 @@
         <v>1.25</v>
       </c>
       <c r="C2" t="n">
-        <v>1294</v>
+        <v>628</v>
       </c>
       <c r="D2" t="n">
-        <v>448</v>
+        <v>204</v>
       </c>
       <c r="E2" t="n">
-        <v>863</v>
+        <v>372</v>
       </c>
       <c r="F2" t="n">
-        <v>428</v>
+        <v>101</v>
       </c>
       <c r="G2" t="n">
-        <v>9.821889746119265</v>
+        <v>6.248384315287693</v>
       </c>
       <c r="H2" t="n">
-        <v>44.98392105742823</v>
+        <v>22.88855323498137</v>
       </c>
       <c r="I2" t="n">
-        <v>0.3033336062217092</v>
+        <v>0.1999325356446183</v>
       </c>
       <c r="J2" t="n">
-        <v>0.6132042327662889</v>
+        <v>0.3282759441062785</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>347.5625</v>
       </c>
       <c r="L2" t="n">
         <v>0.8333333333333334</v>
@@ -1594,31 +1594,31 @@
         <v>1.25</v>
       </c>
       <c r="C3" t="n">
-        <v>1332</v>
+        <v>624</v>
       </c>
       <c r="D3" t="n">
-        <v>377</v>
+        <v>189</v>
       </c>
       <c r="E3" t="n">
-        <v>793</v>
+        <v>344</v>
       </c>
       <c r="F3" t="n">
-        <v>395</v>
+        <v>99</v>
       </c>
       <c r="G3" t="n">
-        <v>31.42453185888007</v>
+        <v>14.05331117496826</v>
       </c>
       <c r="H3" t="n">
-        <v>106.0888671710854</v>
+        <v>53.81865542591549</v>
       </c>
       <c r="I3" t="n">
-        <v>1.237932218820784</v>
+        <v>0.3311244177166348</v>
       </c>
       <c r="J3" t="n">
-        <v>3.002654192037877</v>
+        <v>0.6870031729340532</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>425.40234375</v>
       </c>
       <c r="L3" t="n">
         <v>0.625</v>
@@ -1632,31 +1632,31 @@
         <v>1.25</v>
       </c>
       <c r="C4" t="n">
-        <v>1364</v>
+        <v>626</v>
       </c>
       <c r="D4" t="n">
-        <v>300</v>
+        <v>157</v>
       </c>
       <c r="E4" t="n">
-        <v>720</v>
+        <v>291</v>
       </c>
       <c r="F4" t="n">
-        <v>322</v>
+        <v>57</v>
       </c>
       <c r="G4" t="n">
-        <v>95.48772080696654</v>
+        <v>47.88645441434346</v>
       </c>
       <c r="H4" t="n">
-        <v>324.3207123058382</v>
+        <v>171.6732608885504</v>
       </c>
       <c r="I4" t="n">
-        <v>2.315151128917929</v>
+        <v>1.231310550589112</v>
       </c>
       <c r="J4" t="n">
-        <v>3.523827695287761</v>
+        <v>1.923729777568949</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>705.30859375</v>
       </c>
       <c r="L4" t="n">
         <v>0.4166666666666667</v>
@@ -1670,31 +1670,31 @@
         <v>1.25</v>
       </c>
       <c r="C5" t="n">
-        <v>1379</v>
+        <v>645</v>
       </c>
       <c r="D5" t="n">
-        <v>389</v>
+        <v>146</v>
       </c>
       <c r="E5" t="n">
-        <v>756</v>
+        <v>282</v>
       </c>
       <c r="F5" t="n">
-        <v>335</v>
+        <v>53</v>
       </c>
       <c r="G5" t="n">
-        <v>230.8864183764672</v>
+        <v>125.8319669337943</v>
       </c>
       <c r="H5" t="n">
-        <v>781.3497064244002</v>
+        <v>430.5152797668707</v>
       </c>
       <c r="I5" t="n">
-        <v>6.976126162568104</v>
+        <v>3.153704416472463</v>
       </c>
       <c r="J5" t="n">
-        <v>10.18289490428287</v>
+        <v>5.156607423676176</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>1268.58203125</v>
       </c>
       <c r="L5" t="n">
         <v>0.3125</v>
@@ -1784,31 +1784,31 @@
         <v>2.5</v>
       </c>
       <c r="C2" t="n">
-        <v>843</v>
+        <v>371</v>
       </c>
       <c r="D2" t="n">
-        <v>300</v>
+        <v>140</v>
       </c>
       <c r="E2" t="n">
-        <v>600</v>
+        <v>265</v>
       </c>
       <c r="F2" t="n">
-        <v>320</v>
+        <v>77</v>
       </c>
       <c r="G2" t="n">
-        <v>6.060898373951203</v>
+        <v>3.654186177533119</v>
       </c>
       <c r="H2" t="n">
-        <v>31.13582435471471</v>
+        <v>16.40369262150489</v>
       </c>
       <c r="I2" t="n">
-        <v>0.2247232985682766</v>
+        <v>0.1341939615085706</v>
       </c>
       <c r="J2" t="n">
-        <v>0.6057792662177215</v>
+        <v>0.1978606728371219</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>347.5625</v>
       </c>
       <c r="L2" t="n">
         <v>0.8333333333333334</v>
@@ -1822,31 +1822,31 @@
         <v>2.5</v>
       </c>
       <c r="C3" t="n">
-        <v>879</v>
+        <v>382</v>
       </c>
       <c r="D3" t="n">
-        <v>270</v>
+        <v>119</v>
       </c>
       <c r="E3" t="n">
-        <v>557</v>
+        <v>247</v>
       </c>
       <c r="F3" t="n">
-        <v>296</v>
+        <v>73</v>
       </c>
       <c r="G3" t="n">
-        <v>49.02228045230731</v>
+        <v>9.385341643821448</v>
       </c>
       <c r="H3" t="n">
-        <v>89.71595810016152</v>
+        <v>37.66826786636375</v>
       </c>
       <c r="I3" t="n">
-        <v>8.099671813426539</v>
+        <v>0.2593262505251905</v>
       </c>
       <c r="J3" t="n">
-        <v>14.20752278342843</v>
+        <v>0.4747780929319549</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>425.40234375</v>
       </c>
       <c r="L3" t="n">
         <v>0.625</v>
@@ -1860,31 +1860,31 @@
         <v>2.5</v>
       </c>
       <c r="C4" t="n">
-        <v>879</v>
+        <v>382</v>
       </c>
       <c r="D4" t="n">
-        <v>285</v>
+        <v>101</v>
       </c>
       <c r="E4" t="n">
-        <v>572</v>
+        <v>220</v>
       </c>
       <c r="F4" t="n">
-        <v>286</v>
+        <v>65</v>
       </c>
       <c r="G4" t="n">
-        <v>61.62499541416764</v>
+        <v>32.78437312971801</v>
       </c>
       <c r="H4" t="n">
-        <v>222.6805510720005</v>
+        <v>120.3712185136974</v>
       </c>
       <c r="I4" t="n">
-        <v>1.673721309634855</v>
+        <v>0.7142942612990724</v>
       </c>
       <c r="J4" t="n">
-        <v>2.512818780844098</v>
+        <v>1.301621933234854</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>705.30859375</v>
       </c>
       <c r="L4" t="n">
         <v>0.4166666666666667</v>
@@ -1898,31 +1898,31 @@
         <v>2.5</v>
       </c>
       <c r="C5" t="n">
-        <v>895</v>
+        <v>394</v>
       </c>
       <c r="D5" t="n">
-        <v>224</v>
+        <v>117</v>
       </c>
       <c r="E5" t="n">
-        <v>456</v>
+        <v>249</v>
       </c>
       <c r="F5" t="n">
-        <v>234</v>
+        <v>65</v>
       </c>
       <c r="G5" t="n">
-        <v>151.8492981974268</v>
+        <v>80.74988319212571</v>
       </c>
       <c r="H5" t="n">
-        <v>506.1342428829521</v>
+        <v>288.3058122112416</v>
       </c>
       <c r="I5" t="n">
-        <v>4.39692868827842</v>
+        <v>2.365673603722825</v>
       </c>
       <c r="J5" t="n">
-        <v>7.157999571063554</v>
+        <v>3.756237500347196</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>1261.7890625</v>
       </c>
       <c r="L5" t="n">
         <v>0.3125</v>
@@ -2012,31 +2012,31 @@
         <v>5</v>
       </c>
       <c r="C2" t="n">
-        <v>663</v>
+        <v>253</v>
       </c>
       <c r="D2" t="n">
-        <v>257</v>
+        <v>110</v>
       </c>
       <c r="E2" t="n">
-        <v>503</v>
+        <v>212</v>
       </c>
       <c r="F2" t="n">
-        <v>306</v>
+        <v>72</v>
       </c>
       <c r="G2" t="n">
-        <v>4.855142531567253</v>
+        <v>2.663567811017856</v>
       </c>
       <c r="H2" t="n">
-        <v>26.38950642675627</v>
+        <v>12.02881676633842</v>
       </c>
       <c r="I2" t="n">
-        <v>0.209309325669891</v>
+        <v>0.0841014643665397</v>
       </c>
       <c r="J2" t="n">
-        <v>0.3106209954712528</v>
+        <v>0.1479429709725076</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>347.5625</v>
       </c>
       <c r="L2" t="n">
         <v>0.8333333333333334</v>
@@ -2050,31 +2050,31 @@
         <v>5</v>
       </c>
       <c r="C3" t="n">
-        <v>708</v>
+        <v>258</v>
       </c>
       <c r="D3" t="n">
-        <v>283</v>
+        <v>100</v>
       </c>
       <c r="E3" t="n">
-        <v>539</v>
+        <v>198</v>
       </c>
       <c r="F3" t="n">
-        <v>315</v>
+        <v>61</v>
       </c>
       <c r="G3" t="n">
-        <v>16.07347918546293</v>
+        <v>6.659149925690144</v>
       </c>
       <c r="H3" t="n">
-        <v>59.32980544108432</v>
+        <v>27.86360370786861</v>
       </c>
       <c r="I3" t="n">
-        <v>0.4451761174714183</v>
+        <v>0.1702842828817661</v>
       </c>
       <c r="J3" t="n">
-        <v>0.8718546741874879</v>
+        <v>0.4087435747496777</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>425.40234375</v>
       </c>
       <c r="L3" t="n">
         <v>0.625</v>
@@ -2088,31 +2088,31 @@
         <v>5</v>
       </c>
       <c r="C4" t="n">
-        <v>711</v>
+        <v>248</v>
       </c>
       <c r="D4" t="n">
-        <v>221</v>
+        <v>94</v>
       </c>
       <c r="E4" t="n">
-        <v>438</v>
+        <v>202</v>
       </c>
       <c r="F4" t="n">
-        <v>240</v>
+        <v>57</v>
       </c>
       <c r="G4" t="n">
-        <v>50.47467044508085</v>
+        <v>23.21078818035312</v>
       </c>
       <c r="H4" t="n">
-        <v>180.8124203648185</v>
+        <v>89.90002425131388</v>
       </c>
       <c r="I4" t="n">
-        <v>1.405742380884475</v>
+        <v>0.7171471484471106</v>
       </c>
       <c r="J4" t="n">
-        <v>2.074586911941878</v>
+        <v>0.8442013307940209</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>702.2421875</v>
       </c>
       <c r="L4" t="n">
         <v>0.4166666666666667</v>
@@ -2126,31 +2126,31 @@
         <v>5</v>
       </c>
       <c r="C5" t="n">
-        <v>720</v>
+        <v>248</v>
       </c>
       <c r="D5" t="n">
-        <v>175</v>
+        <v>73</v>
       </c>
       <c r="E5" t="n">
-        <v>373</v>
+        <v>165</v>
       </c>
       <c r="F5" t="n">
-        <v>209</v>
+        <v>43</v>
       </c>
       <c r="G5" t="n">
-        <v>120.5373222955968</v>
+        <v>56.83620678074658</v>
       </c>
       <c r="H5" t="n">
-        <v>399.3175338545116</v>
+        <v>204.5307487079408</v>
       </c>
       <c r="I5" t="n">
-        <v>3.439200316788628</v>
+        <v>1.766409808304161</v>
       </c>
       <c r="J5" t="n">
-        <v>5.522909677354619</v>
+        <v>2.693274196702987</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>1255.453125</v>
       </c>
       <c r="L5" t="n">
         <v>0.3125</v>
@@ -2240,31 +2240,31 @@
         <v>10</v>
       </c>
       <c r="C2" t="n">
-        <v>619</v>
+        <v>194</v>
       </c>
       <c r="D2" t="n">
-        <v>285</v>
+        <v>93</v>
       </c>
       <c r="E2" t="n">
-        <v>522</v>
+        <v>151</v>
       </c>
       <c r="F2" t="n">
-        <v>345</v>
+        <v>62</v>
       </c>
       <c r="G2" t="n">
-        <v>4.822351032635197</v>
+        <v>1.925949798664078</v>
       </c>
       <c r="H2" t="n">
-        <v>22.0270862741163</v>
+        <v>7.403968306956813</v>
       </c>
       <c r="I2" t="n">
-        <v>0.1696899380767713</v>
+        <v>0.06508247484452989</v>
       </c>
       <c r="J2" t="n">
-        <v>0.271674955496564</v>
+        <v>0.0847447603009638</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>344.86328125</v>
       </c>
       <c r="L2" t="n">
         <v>0.8333333333333334</v>
@@ -2278,31 +2278,31 @@
         <v>10</v>
       </c>
       <c r="C3" t="n">
-        <v>666</v>
+        <v>194</v>
       </c>
       <c r="D3" t="n">
-        <v>267</v>
+        <v>95</v>
       </c>
       <c r="E3" t="n">
-        <v>493</v>
+        <v>136</v>
       </c>
       <c r="F3" t="n">
-        <v>320</v>
+        <v>66</v>
       </c>
       <c r="G3" t="n">
-        <v>13.98868884670082</v>
+        <v>4.360094435047358</v>
       </c>
       <c r="H3" t="n">
-        <v>52.53486259514466</v>
+        <v>18.34872942650691</v>
       </c>
       <c r="I3" t="n">
-        <v>0.5419181052129711</v>
+        <v>0.1380650654900817</v>
       </c>
       <c r="J3" t="n">
-        <v>0.9414641577750441</v>
+        <v>0.1610804649535564</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>425.40234375</v>
       </c>
       <c r="L3" t="n">
         <v>0.625</v>
@@ -2316,31 +2316,31 @@
         <v>10</v>
       </c>
       <c r="C4" t="n">
-        <v>664</v>
+        <v>202</v>
       </c>
       <c r="D4" t="n">
-        <v>207</v>
+        <v>69</v>
       </c>
       <c r="E4" t="n">
-        <v>404</v>
+        <v>136</v>
       </c>
       <c r="F4" t="n">
-        <v>263</v>
+        <v>51</v>
       </c>
       <c r="G4" t="n">
-        <v>45.33196399139706</v>
+        <v>15.23244327539578</v>
       </c>
       <c r="H4" t="n">
-        <v>163.0275517153786</v>
+        <v>55.24015376134776</v>
       </c>
       <c r="I4" t="n">
-        <v>1.280679006013088</v>
+        <v>0.3628585792612282</v>
       </c>
       <c r="J4" t="n">
-        <v>2.023490183171816</v>
+        <v>0.5470570668112484</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>700.08984375</v>
       </c>
       <c r="L4" t="n">
         <v>0.4166666666666667</v>
@@ -2354,31 +2354,31 @@
         <v>10</v>
       </c>
       <c r="C5" t="n">
-        <v>675</v>
+        <v>201</v>
       </c>
       <c r="D5" t="n">
-        <v>213</v>
+        <v>64</v>
       </c>
       <c r="E5" t="n">
-        <v>423</v>
+        <v>123</v>
       </c>
       <c r="F5" t="n">
-        <v>271</v>
+        <v>37</v>
       </c>
       <c r="G5" t="n">
-        <v>111.568812348647</v>
+        <v>37.10530396830291</v>
       </c>
       <c r="H5" t="n">
-        <v>383.76236356562</v>
+        <v>130.0768073198851</v>
       </c>
       <c r="I5" t="n">
-        <v>3.66077060427051</v>
+        <v>1.096488550305366</v>
       </c>
       <c r="J5" t="n">
-        <v>5.478542647440918</v>
+        <v>1.593927752226591</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>1255.41796875</v>
       </c>
       <c r="L5" t="n">
         <v>0.3125</v>
@@ -2468,31 +2468,31 @@
         <v>20</v>
       </c>
       <c r="C2" t="n">
-        <v>697</v>
+        <v>134</v>
       </c>
       <c r="D2" t="n">
-        <v>325</v>
+        <v>71</v>
       </c>
       <c r="E2" t="n">
-        <v>614</v>
+        <v>107</v>
       </c>
       <c r="F2" t="n">
-        <v>416</v>
+        <v>55</v>
       </c>
       <c r="G2" t="n">
-        <v>5.375350917107426</v>
+        <v>1.071887104073539</v>
       </c>
       <c r="H2" t="n">
-        <v>26.16464210103732</v>
+        <v>5.242887788219377</v>
       </c>
       <c r="I2" t="n">
-        <v>0.3241760305827481</v>
+        <v>0.0434046026784926</v>
       </c>
       <c r="J2" t="n">
-        <v>0.3905542844440787</v>
+        <v>0.0731638579163699</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>339.6953125</v>
       </c>
       <c r="L2" t="n">
         <v>0.8333333333333334</v>
@@ -2506,31 +2506,31 @@
         <v>20</v>
       </c>
       <c r="C3" t="n">
-        <v>711</v>
+        <v>135</v>
       </c>
       <c r="D3" t="n">
-        <v>260</v>
+        <v>64</v>
       </c>
       <c r="E3" t="n">
-        <v>516</v>
+        <v>105</v>
       </c>
       <c r="F3" t="n">
-        <v>365</v>
+        <v>47</v>
       </c>
       <c r="G3" t="n">
-        <v>15.22564096085262</v>
+        <v>2.825710028875619</v>
       </c>
       <c r="H3" t="n">
-        <v>60.20525390375406</v>
+        <v>11.78791014919989</v>
       </c>
       <c r="I3" t="n">
-        <v>0.4884560155915094</v>
+        <v>0.0634014257229862</v>
       </c>
       <c r="J3" t="n">
-        <v>0.8185585525352506</v>
+        <v>0.1414963684510438</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>414.5625</v>
       </c>
       <c r="L3" t="n">
         <v>0.625</v>
@@ -2544,31 +2544,31 @@
         <v>20</v>
       </c>
       <c r="C4" t="n">
-        <v>705</v>
+        <v>135</v>
       </c>
       <c r="D4" t="n">
-        <v>257</v>
+        <v>49</v>
       </c>
       <c r="E4" t="n">
-        <v>497</v>
+        <v>92</v>
       </c>
       <c r="F4" t="n">
-        <v>332</v>
+        <v>36</v>
       </c>
       <c r="G4" t="n">
-        <v>49.61684343672823</v>
+        <v>9.631501971744001</v>
       </c>
       <c r="H4" t="n">
-        <v>178.2478612159612</v>
+        <v>35.28778052190319</v>
       </c>
       <c r="I4" t="n">
-        <v>1.849834322696552</v>
+        <v>0.2344712219201027</v>
       </c>
       <c r="J4" t="n">
-        <v>2.918105075834319</v>
+        <v>0.3917439859360456</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>687.6484375</v>
       </c>
       <c r="L4" t="n">
         <v>0.4166666666666667</v>
@@ -2582,31 +2582,31 @@
         <v>20</v>
       </c>
       <c r="C5" t="n">
-        <v>709</v>
+        <v>138</v>
       </c>
       <c r="D5" t="n">
-        <v>253</v>
+        <v>50</v>
       </c>
       <c r="E5" t="n">
-        <v>506</v>
+        <v>74</v>
       </c>
       <c r="F5" t="n">
-        <v>348</v>
+        <v>36</v>
       </c>
       <c r="G5" t="n">
-        <v>115.8653817678569</v>
+        <v>23.73199123726226</v>
       </c>
       <c r="H5" t="n">
-        <v>405.7470981484512</v>
+        <v>83.02786784479395</v>
       </c>
       <c r="I5" t="n">
-        <v>4.20810675714165</v>
+        <v>0.6523936265148222</v>
       </c>
       <c r="J5" t="n">
-        <v>5.84556619275827</v>
+        <v>1.07542175007984</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>1215.41796875</v>
       </c>
       <c r="L5" t="n">
         <v>0.3125</v>
@@ -2648,10 +2648,10 @@
         <v>20</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0001709991969209013</v>
+        <v>6.861913985167839e-05</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0003203688486081723</v>
+        <v>2.009867824102167e-05</v>
       </c>
     </row>
     <row r="3">
@@ -2659,10 +2659,10 @@
         <v>10</v>
       </c>
       <c r="B3" t="n">
-        <v>0.0001559881317997365</v>
+        <v>3.614480414538668e-05</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0002515592355026354</v>
+        <v>1.058641934152947e-05</v>
       </c>
     </row>
     <row r="4">
@@ -2670,10 +2670,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.0001347587219089792</v>
+        <v>1.859626917557472e-05</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0001912535029975272</v>
+        <v>5.454808593150901e-06</v>
       </c>
     </row>
     <row r="5">
@@ -2681,10 +2681,10 @@
         <v>2.5</v>
       </c>
       <c r="B5" t="n">
-        <v>0.0001010630307492901</v>
+        <v>9.435950570634227e-06</v>
       </c>
       <c r="C5" t="n">
-        <v>0.00012932230543864</v>
+        <v>2.769208814581154e-06</v>
       </c>
     </row>
   </sheetData>
@@ -2723,10 +2723,10 @@
         <v>20</v>
       </c>
       <c r="B2" t="n">
-        <v>2.98496374515378</v>
+        <v>0.3907703017006184</v>
       </c>
       <c r="C2" t="n">
-        <v>3.040199587100684</v>
+        <v>0.08880216201293692</v>
       </c>
     </row>
     <row r="3">
@@ -2734,10 +2734,10 @@
         <v>10</v>
       </c>
       <c r="B3" t="n">
-        <v>2.45130301380839</v>
+        <v>0.2189032099578059</v>
       </c>
       <c r="C3" t="n">
-        <v>2.023765220652393</v>
+        <v>0.05040082844697263</v>
       </c>
     </row>
     <row r="4">
@@ -2745,10 +2745,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="n">
-        <v>1.867981830862222</v>
+        <v>0.1166657843076625</v>
       </c>
       <c r="C4" t="n">
-        <v>1.294520303615035</v>
+        <v>0.02718916884395936</v>
       </c>
     </row>
     <row r="5">
@@ -2756,10 +2756,10 @@
         <v>2.5</v>
       </c>
       <c r="B5" t="n">
-        <v>1.210050303823538</v>
+        <v>0.06028317796433912</v>
       </c>
       <c r="C5" t="n">
-        <v>0.7522473795820617</v>
+        <v>0.01416114467481035</v>
       </c>
     </row>
   </sheetData>
@@ -2798,10 +2798,10 @@
         <v>20</v>
       </c>
       <c r="B2" t="n">
-        <v>1.449148545186773</v>
+        <v>0.5970558168397988</v>
       </c>
       <c r="C2" t="n">
-        <v>0.5254194996951481</v>
+        <v>0.5142946966708221</v>
       </c>
     </row>
     <row r="3">
@@ -2809,10 +2809,10 @@
         <v>10</v>
       </c>
       <c r="B3" t="n">
-        <v>0.7431859716459603</v>
+        <v>0.4149848573243486</v>
       </c>
       <c r="C3" t="n">
-        <v>0.276974579439873</v>
+        <v>0.3224294258532335</v>
       </c>
     </row>
     <row r="4">
@@ -2820,10 +2820,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.384988400928016</v>
+        <v>0.2644009348350175</v>
       </c>
       <c r="C4" t="n">
-        <v>0.3226619041973237</v>
+        <v>0.1898389581894845</v>
       </c>
     </row>
     <row r="5">
@@ -2831,10 +2831,10 @@
         <v>2.5</v>
       </c>
       <c r="B5" t="n">
-        <v>0.294695801695866</v>
+        <v>0.1501191698936636</v>
       </c>
       <c r="C5" t="n">
-        <v>0.2931091085711133</v>
+        <v>0.1046185251248387</v>
       </c>
     </row>
   </sheetData>
@@ -2873,10 +2873,10 @@
         <v>20</v>
       </c>
       <c r="B2" t="n">
-        <v>1.533563486252732</v>
+        <v>0.7262156452315093</v>
       </c>
       <c r="C2" t="n">
-        <v>0.2259814560460624</v>
+        <v>0.1792683374659095</v>
       </c>
     </row>
     <row r="3">
@@ -2884,10 +2884,10 @@
         <v>10</v>
       </c>
       <c r="B3" t="n">
-        <v>0.8087422661684079</v>
+        <v>0.3873553307000035</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1579359208736714</v>
+        <v>0.09896650633460986</v>
       </c>
     </row>
     <row r="4">
@@ -2895,10 +2895,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.4223994900082316</v>
+        <v>0.2002905934369001</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1145604784899013</v>
+        <v>0.05210574747214979</v>
       </c>
     </row>
     <row r="5">
@@ -2906,10 +2906,10 @@
         <v>2.5</v>
       </c>
       <c r="B5" t="n">
-        <v>0.2181060347599121</v>
+        <v>0.1018664672225554</v>
       </c>
       <c r="C5" t="n">
-        <v>0.07110271600778782</v>
+        <v>0.02673744943294221</v>
       </c>
     </row>
   </sheetData>
@@ -2956,10 +2956,10 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="C2" t="n">
-        <v>0.3823674973288085</v>
+        <v>0.9432299482861873</v>
       </c>
       <c r="D2" t="n">
-        <v>1.506856388605617</v>
+        <v>3.442230948793381</v>
       </c>
     </row>
     <row r="3">
@@ -2970,10 +2970,10 @@
         <v>0.625</v>
       </c>
       <c r="C3" t="n">
-        <v>0.2697994726898928</v>
+        <v>0.7157432785232639</v>
       </c>
       <c r="D3" t="n">
-        <v>1.107563704922098</v>
+        <v>2.867512999269279</v>
       </c>
     </row>
     <row r="4">
@@ -2984,10 +2984,10 @@
         <v>0.4166666666666667</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1165894742843467</v>
+        <v>0.3090874467158319</v>
       </c>
       <c r="D4" t="n">
-        <v>0.9978358619454448</v>
+        <v>2.604943797498385</v>
       </c>
     </row>
   </sheetData>
@@ -3026,10 +3026,10 @@
         <v>20</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0001594622950021406</v>
+        <v>6.859932679041263e-05</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0003373914004073319</v>
+        <v>2.44307608736606e-05</v>
       </c>
     </row>
     <row r="3">
@@ -3037,10 +3037,10 @@
         <v>10</v>
       </c>
       <c r="B3" t="n">
-        <v>0.0001522218107619859</v>
+        <v>3.612326492624447e-05</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0002817171478283104</v>
+        <v>1.289065287278472e-05</v>
       </c>
     </row>
     <row r="4">
@@ -3048,10 +3048,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.0001334937345640079</v>
+        <v>1.858552620997826e-05</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0002149395379653581</v>
+        <v>6.647807413853865e-06</v>
       </c>
     </row>
     <row r="5">
@@ -3059,10 +3059,10 @@
         <v>2.5</v>
       </c>
       <c r="B5" t="n">
-        <v>0.0001002805548032077</v>
+        <v>9.429494143013041e-06</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0001440764717680095</v>
+        <v>3.375182154053831e-06</v>
       </c>
     </row>
   </sheetData>
@@ -3101,10 +3101,10 @@
         <v>20</v>
       </c>
       <c r="B2" t="n">
-        <v>2.805211181707069</v>
+        <v>0.386440036671197</v>
       </c>
       <c r="C2" t="n">
-        <v>3.119106005016937</v>
+        <v>0.09528265790510274</v>
       </c>
     </row>
     <row r="3">
@@ -3112,10 +3112,10 @@
         <v>10</v>
       </c>
       <c r="B3" t="n">
-        <v>2.429343868670993</v>
+        <v>0.2162373732711009</v>
       </c>
       <c r="C3" t="n">
-        <v>2.227664726592091</v>
+        <v>0.05426407555529993</v>
       </c>
     </row>
     <row r="4">
@@ -3123,10 +3123,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="n">
-        <v>1.881407768848816</v>
+        <v>0.1152479717962462</v>
       </c>
       <c r="C4" t="n">
-        <v>1.407151832439923</v>
+        <v>0.02927925515700906</v>
       </c>
     </row>
     <row r="5">
@@ -3134,10 +3134,10 @@
         <v>2.5</v>
       </c>
       <c r="B5" t="n">
-        <v>1.222850852461482</v>
+        <v>0.05951718760139807</v>
       </c>
       <c r="C5" t="n">
-        <v>0.8073571820966245</v>
+        <v>0.01522878299834563</v>
       </c>
     </row>
   </sheetData>
@@ -3176,10 +3176,10 @@
         <v>20</v>
       </c>
       <c r="B2" t="n">
-        <v>1.484416573807954</v>
+        <v>0.5992633038849854</v>
       </c>
       <c r="C2" t="n">
-        <v>0.5325738929019586</v>
+        <v>0.5384945500984957</v>
       </c>
     </row>
     <row r="3">
@@ -3187,10 +3187,10 @@
         <v>10</v>
       </c>
       <c r="B3" t="n">
-        <v>0.782370477593142</v>
+        <v>0.4042157641730316</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3047882044685506</v>
+        <v>0.3363601949528302</v>
       </c>
     </row>
     <row r="4">
@@ -3198,10 +3198,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.4031764862152093</v>
+        <v>0.2561172004125861</v>
       </c>
       <c r="C4" t="n">
-        <v>0.3535094614371481</v>
+        <v>0.1984389081789122</v>
       </c>
     </row>
     <row r="5">
@@ -3209,10 +3209,10 @@
         <v>2.5</v>
       </c>
       <c r="B5" t="n">
-        <v>0.2874660160622931</v>
+        <v>0.1451961060586809</v>
       </c>
       <c r="C5" t="n">
-        <v>0.309374377880899</v>
+        <v>0.109527318571258</v>
       </c>
     </row>
   </sheetData>
@@ -3251,10 +3251,10 @@
         <v>20</v>
       </c>
       <c r="B2" t="n">
-        <v>1.539143209603697</v>
+        <v>0.7308078449784603</v>
       </c>
       <c r="C2" t="n">
-        <v>0.2511532860535337</v>
+        <v>0.1906305489920335</v>
       </c>
     </row>
     <row r="3">
@@ -3262,10 +3262,10 @@
         <v>10</v>
       </c>
       <c r="B3" t="n">
-        <v>0.8138917731028882</v>
+        <v>0.389931109599556</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1809413716421074</v>
+        <v>0.105431531068792</v>
       </c>
     </row>
     <row r="4">
@@ -3273,10 +3273,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.4267650146441356</v>
+        <v>0.2016703587766013</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1297642264124254</v>
+        <v>0.05560254675614665</v>
       </c>
     </row>
     <row r="5">
@@ -3284,10 +3284,10 @@
         <v>2.5</v>
       </c>
       <c r="B5" t="n">
-        <v>0.2214844448343721</v>
+        <v>0.1025854490942421</v>
       </c>
       <c r="C5" t="n">
-        <v>0.08166563705684815</v>
+        <v>0.0285651294638763</v>
       </c>
     </row>
   </sheetData>
@@ -3326,10 +3326,10 @@
         <v>20</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0001557405283033984</v>
+        <v>6.85171551595402e-05</v>
       </c>
       <c r="C2" t="n">
-        <v>0.000368368442655705</v>
+        <v>3.16365690949549e-05</v>
       </c>
     </row>
     <row r="3">
@@ -3337,10 +3337,10 @@
         <v>10</v>
       </c>
       <c r="B3" t="n">
-        <v>0.0001487027880044313</v>
+        <v>3.6085740405188e-05</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0003102419222063683</v>
+        <v>1.674011918658863e-05</v>
       </c>
     </row>
     <row r="4">
@@ -3348,10 +3348,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.0001323713624135571</v>
+        <v>1.856658659326058e-05</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0002424174455241145</v>
+        <v>8.645823692933431e-06</v>
       </c>
     </row>
     <row r="5">
@@ -3359,10 +3359,10 @@
         <v>2.5</v>
       </c>
       <c r="B5" t="n">
-        <v>0.0001000474416469423</v>
+        <v>9.418511884875625e-06</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0001620948283219687</v>
+        <v>4.399097612771916e-06</v>
       </c>
     </row>
   </sheetData>
@@ -3401,10 +3401,10 @@
         <v>20</v>
       </c>
       <c r="B2" t="n">
-        <v>2.720426873844048</v>
+        <v>0.3827267142891916</v>
       </c>
       <c r="C2" t="n">
-        <v>3.20862867884727</v>
+        <v>0.1024494230205506</v>
       </c>
     </row>
     <row r="3">
@@ -3412,10 +3412,10 @@
         <v>10</v>
       </c>
       <c r="B3" t="n">
-        <v>2.408334686115457</v>
+        <v>0.2140907215949031</v>
       </c>
       <c r="C3" t="n">
-        <v>2.343498911518935</v>
+        <v>0.05843563168868448</v>
       </c>
     </row>
     <row r="4">
@@ -3423,10 +3423,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="n">
-        <v>1.893253536936866</v>
+        <v>0.1140772870481497</v>
       </c>
       <c r="C4" t="n">
-        <v>1.487709479262696</v>
+        <v>0.03157849791112619</v>
       </c>
     </row>
     <row r="5">
@@ -3434,10 +3434,10 @@
         <v>2.5</v>
       </c>
       <c r="B5" t="n">
-        <v>1.237102233681117</v>
+        <v>0.05889861064676413</v>
       </c>
       <c r="C5" t="n">
-        <v>0.8533735301519084</v>
+        <v>0.01650958911224861</v>
       </c>
     </row>
   </sheetData>
@@ -3476,10 +3476,10 @@
         <v>20</v>
       </c>
       <c r="B2" t="n">
-        <v>1.516407094901761</v>
+        <v>0.6052248592972028</v>
       </c>
       <c r="C2" t="n">
-        <v>0.5805133444088015</v>
+        <v>0.5895512371001149</v>
       </c>
     </row>
     <row r="3">
@@ -3487,10 +3487,10 @@
         <v>10</v>
       </c>
       <c r="B3" t="n">
-        <v>0.8129396999824045</v>
+        <v>0.4001445832613257</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3404117922346541</v>
+        <v>0.3687145035079033</v>
       </c>
     </row>
     <row r="4">
@@ -3498,10 +3498,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.4203783626447944</v>
+        <v>0.25225228770318</v>
       </c>
       <c r="C4" t="n">
-        <v>0.390762873678442</v>
+        <v>0.2174186924310594</v>
       </c>
     </row>
     <row r="5">
@@ -3509,10 +3509,10 @@
         <v>2.5</v>
       </c>
       <c r="B5" t="n">
-        <v>0.2873984528038677</v>
+        <v>0.1429504584042143</v>
       </c>
       <c r="C5" t="n">
-        <v>0.3328266255582831</v>
+        <v>0.1200915381973557</v>
       </c>
     </row>
   </sheetData>
@@ -3551,10 +3551,10 @@
         <v>20</v>
       </c>
       <c r="B2" t="n">
-        <v>1.547661420060854</v>
+        <v>0.7345533900925159</v>
       </c>
       <c r="C2" t="n">
-        <v>0.2835715292952474</v>
+        <v>0.1999657971179189</v>
       </c>
     </row>
     <row r="3">
@@ -3562,10 +3562,10 @@
         <v>10</v>
       </c>
       <c r="B3" t="n">
-        <v>0.8196368277131756</v>
+        <v>0.3921220113336882</v>
       </c>
       <c r="C3" t="n">
-        <v>0.2043836486074038</v>
+        <v>0.1108328466606258</v>
       </c>
     </row>
     <row r="4">
@@ -3573,10 +3573,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.4305798228736171</v>
+        <v>0.2028512500554182</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1436973097499629</v>
+        <v>0.05851041572529476</v>
       </c>
     </row>
     <row r="5">
@@ -3584,10 +3584,10 @@
         <v>2.5</v>
       </c>
       <c r="B5" t="n">
-        <v>0.2252847679815164</v>
+        <v>0.103211713277186</v>
       </c>
       <c r="C5" t="n">
-        <v>0.09293678583818445</v>
+        <v>0.03009662948257975</v>
       </c>
     </row>
   </sheetData>
@@ -3626,10 +3626,10 @@
         <v>20</v>
       </c>
       <c r="B2" t="n">
-        <v>0.0001548577175407237</v>
+        <v>6.847384831557791e-05</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0003880403433765878</v>
+        <v>3.799293189241131e-05</v>
       </c>
     </row>
     <row r="3">
@@ -3637,10 +3637,10 @@
         <v>10</v>
       </c>
       <c r="B3" t="n">
-        <v>0.0001475247523732729</v>
+        <v>3.607008106871551e-05</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0003255191843024404</v>
+        <v>2.012965933879364e-05</v>
       </c>
     </row>
     <row r="4">
@@ -3648,10 +3648,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.0001320793361649934</v>
+        <v>1.855849598931096e-05</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0002565275740252413</v>
+        <v>1.039663723452244e-05</v>
       </c>
     </row>
     <row r="5">
@@ -3659,10 +3659,10 @@
         <v>2.5</v>
       </c>
       <c r="B5" t="n">
-        <v>0.0001001494180043018</v>
+        <v>9.417316719593407e-06</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0001728685743592366</v>
+        <v>5.293952238892421e-06</v>
       </c>
     </row>
   </sheetData>
@@ -3701,10 +3701,10 @@
         <v>20</v>
       </c>
       <c r="B2" t="n">
-        <v>2.693989332131629</v>
+        <v>0.3813443303571009</v>
       </c>
       <c r="C2" t="n">
-        <v>3.247091111239929</v>
+        <v>0.1052036320083347</v>
       </c>
     </row>
     <row r="3">
@@ -3712,10 +3712,10 @@
         <v>10</v>
       </c>
       <c r="B3" t="n">
-        <v>2.403316698591115</v>
+        <v>0.2133683971553762</v>
       </c>
       <c r="C3" t="n">
-        <v>2.387956873234439</v>
+        <v>0.06006755572974963</v>
       </c>
     </row>
     <row r="4">
@@ -3723,10 +3723,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="n">
-        <v>1.898027551169092</v>
+        <v>0.1136570809620425</v>
       </c>
       <c r="C4" t="n">
-        <v>1.518650314840415</v>
+        <v>0.03245198540994086</v>
       </c>
     </row>
     <row r="5">
@@ -3734,10 +3734,10 @@
         <v>2.5</v>
       </c>
       <c r="B5" t="n">
-        <v>1.24428696223744</v>
+        <v>0.05875057884980658</v>
       </c>
       <c r="C5" t="n">
-        <v>0.8717714040608451</v>
+        <v>0.01692817063568447</v>
       </c>
     </row>
   </sheetData>
@@ -3784,10 +3784,10 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="C2" t="n">
-        <v>0.3292808214677116</v>
+        <v>0.3149265090601775</v>
       </c>
       <c r="D2" t="n">
-        <v>1.050545874171268</v>
+        <v>0.8485065978335933</v>
       </c>
     </row>
     <row r="3">
@@ -3798,10 +3798,10 @@
         <v>0.625</v>
       </c>
       <c r="C3" t="n">
-        <v>0.2992005346904201</v>
+        <v>0.2791304185326616</v>
       </c>
       <c r="D3" t="n">
-        <v>0.7516615373077724</v>
+        <v>0.6428603525125465</v>
       </c>
     </row>
     <row r="4">
@@ -3812,10 +3812,10 @@
         <v>0.4166666666666667</v>
       </c>
       <c r="C4" t="n">
-        <v>0.134782445564479</v>
+        <v>0.1219612805758827</v>
       </c>
       <c r="D4" t="n">
-        <v>0.6567162773217535</v>
+        <v>0.55442547398963</v>
       </c>
     </row>
   </sheetData>
@@ -3854,10 +3854,10 @@
         <v>20</v>
       </c>
       <c r="B2" t="n">
-        <v>1.526774021025038</v>
+        <v>0.6082724997080469</v>
       </c>
       <c r="C2" t="n">
-        <v>0.6113160831248095</v>
+        <v>0.6198991881095463</v>
       </c>
     </row>
     <row r="3">
@@ -3865,10 +3865,10 @@
         <v>10</v>
       </c>
       <c r="B3" t="n">
-        <v>0.8234373938462439</v>
+        <v>0.3993311716281594</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3580495101019552</v>
+        <v>0.3882972554451858</v>
       </c>
     </row>
     <row r="4">
@@ -3876,10 +3876,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.4281550100868545</v>
+        <v>0.2511869685068093</v>
       </c>
       <c r="C4" t="n">
-        <v>0.4083954948024071</v>
+        <v>0.2291970684799</v>
       </c>
     </row>
     <row r="5">
@@ -3887,10 +3887,10 @@
         <v>2.5</v>
       </c>
       <c r="B5" t="n">
-        <v>0.2894834766637824</v>
+        <v>0.142561065155641</v>
       </c>
       <c r="C5" t="n">
-        <v>0.3453424048538393</v>
+        <v>0.126861051895881</v>
       </c>
     </row>
   </sheetData>
@@ -3929,10 +3929,10 @@
         <v>20</v>
       </c>
       <c r="B2" t="n">
-        <v>1.551855699616611</v>
+        <v>0.736392841532328</v>
       </c>
       <c r="C2" t="n">
-        <v>0.2983431586869408</v>
+        <v>0.2046117650570699</v>
       </c>
     </row>
     <row r="3">
@@ -3940,10 +3940,10 @@
         <v>10</v>
       </c>
       <c r="B3" t="n">
-        <v>0.8223656995221381</v>
+        <v>0.3932690406570368</v>
       </c>
       <c r="C3" t="n">
-        <v>0.2146476333336718</v>
+        <v>0.1136682930611382</v>
       </c>
     </row>
     <row r="4">
@@ -3951,10 +3951,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.4321464189059182</v>
+        <v>0.2034819955962572</v>
       </c>
       <c r="C4" t="n">
-        <v>0.149423900949022</v>
+        <v>0.06006210270657932</v>
       </c>
     </row>
     <row r="5">
@@ -3962,10 +3962,10 @@
         <v>2.5</v>
       </c>
       <c r="B5" t="n">
-        <v>0.2269732541009904</v>
+        <v>0.103554849003709</v>
       </c>
       <c r="C5" t="n">
-        <v>0.09773722862299955</v>
+        <v>0.03093173828141062</v>
       </c>
     </row>
   </sheetData>
@@ -4047,31 +4047,31 @@
         <v>20</v>
       </c>
       <c r="C2" t="n">
-        <v>697</v>
+        <v>134</v>
       </c>
       <c r="D2" t="n">
-        <v>325</v>
+        <v>71</v>
       </c>
       <c r="E2" t="n">
-        <v>614</v>
+        <v>107</v>
       </c>
       <c r="F2" t="n">
-        <v>416</v>
+        <v>55</v>
       </c>
       <c r="G2" t="n">
-        <v>5.375350917107426</v>
+        <v>1.071887104073539</v>
       </c>
       <c r="H2" t="n">
-        <v>26.16464210103732</v>
+        <v>5.242887788219377</v>
       </c>
       <c r="I2" t="n">
-        <v>0.3241760305827481</v>
+        <v>0.0434046026784926</v>
       </c>
       <c r="J2" t="n">
-        <v>0.3905542844440787</v>
+        <v>0.0731638579163699</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>339.6953125</v>
       </c>
     </row>
     <row r="3">
@@ -4082,31 +4082,31 @@
         <v>10</v>
       </c>
       <c r="C3" t="n">
-        <v>619</v>
+        <v>194</v>
       </c>
       <c r="D3" t="n">
-        <v>285</v>
+        <v>93</v>
       </c>
       <c r="E3" t="n">
-        <v>522</v>
+        <v>151</v>
       </c>
       <c r="F3" t="n">
-        <v>345</v>
+        <v>62</v>
       </c>
       <c r="G3" t="n">
-        <v>4.822351032635197</v>
+        <v>1.925949798664078</v>
       </c>
       <c r="H3" t="n">
-        <v>22.0270862741163</v>
+        <v>7.403968306956813</v>
       </c>
       <c r="I3" t="n">
-        <v>0.1696899380767713</v>
+        <v>0.06508247484452989</v>
       </c>
       <c r="J3" t="n">
-        <v>0.271674955496564</v>
+        <v>0.0847447603009638</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>344.86328125</v>
       </c>
     </row>
     <row r="4">
@@ -4117,31 +4117,31 @@
         <v>5</v>
       </c>
       <c r="C4" t="n">
-        <v>663</v>
+        <v>253</v>
       </c>
       <c r="D4" t="n">
-        <v>257</v>
+        <v>110</v>
       </c>
       <c r="E4" t="n">
-        <v>503</v>
+        <v>212</v>
       </c>
       <c r="F4" t="n">
-        <v>306</v>
+        <v>72</v>
       </c>
       <c r="G4" t="n">
-        <v>4.855142531567253</v>
+        <v>2.663567811017856</v>
       </c>
       <c r="H4" t="n">
-        <v>26.38950642675627</v>
+        <v>12.02881676633842</v>
       </c>
       <c r="I4" t="n">
-        <v>0.209309325669891</v>
+        <v>0.0841014643665397</v>
       </c>
       <c r="J4" t="n">
-        <v>0.3106209954712528</v>
+        <v>0.1479429709725076</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>347.5625</v>
       </c>
     </row>
     <row r="5">
@@ -4152,31 +4152,31 @@
         <v>2.5</v>
       </c>
       <c r="C5" t="n">
-        <v>843</v>
+        <v>371</v>
       </c>
       <c r="D5" t="n">
-        <v>300</v>
+        <v>140</v>
       </c>
       <c r="E5" t="n">
-        <v>600</v>
+        <v>265</v>
       </c>
       <c r="F5" t="n">
-        <v>320</v>
+        <v>77</v>
       </c>
       <c r="G5" t="n">
-        <v>6.060898373951203</v>
+        <v>3.654186177533119</v>
       </c>
       <c r="H5" t="n">
-        <v>31.13582435471471</v>
+        <v>16.40369262150489</v>
       </c>
       <c r="I5" t="n">
-        <v>0.2247232985682766</v>
+        <v>0.1341939615085706</v>
       </c>
       <c r="J5" t="n">
-        <v>0.6057792662177215</v>
+        <v>0.1978606728371219</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>347.5625</v>
       </c>
     </row>
     <row r="6">
@@ -4187,31 +4187,31 @@
         <v>1.25</v>
       </c>
       <c r="C6" t="n">
-        <v>1294</v>
+        <v>628</v>
       </c>
       <c r="D6" t="n">
-        <v>448</v>
+        <v>204</v>
       </c>
       <c r="E6" t="n">
-        <v>863</v>
+        <v>372</v>
       </c>
       <c r="F6" t="n">
-        <v>428</v>
+        <v>101</v>
       </c>
       <c r="G6" t="n">
-        <v>9.821889746119265</v>
+        <v>6.248384315287693</v>
       </c>
       <c r="H6" t="n">
-        <v>44.98392105742823</v>
+        <v>22.88855323498137</v>
       </c>
       <c r="I6" t="n">
-        <v>0.3033336062217092</v>
+        <v>0.1999325356446183</v>
       </c>
       <c r="J6" t="n">
-        <v>0.6132042327662889</v>
+        <v>0.3282759441062785</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>347.5625</v>
       </c>
     </row>
   </sheetData>
@@ -4293,31 +4293,31 @@
         <v>20</v>
       </c>
       <c r="C2" t="n">
-        <v>711</v>
+        <v>135</v>
       </c>
       <c r="D2" t="n">
-        <v>260</v>
+        <v>64</v>
       </c>
       <c r="E2" t="n">
-        <v>516</v>
+        <v>105</v>
       </c>
       <c r="F2" t="n">
-        <v>365</v>
+        <v>47</v>
       </c>
       <c r="G2" t="n">
-        <v>15.22564096085262</v>
+        <v>2.825710028875619</v>
       </c>
       <c r="H2" t="n">
-        <v>60.20525390375406</v>
+        <v>11.78791014919989</v>
       </c>
       <c r="I2" t="n">
-        <v>0.4884560155915094</v>
+        <v>0.0634014257229862</v>
       </c>
       <c r="J2" t="n">
-        <v>0.8185585525352506</v>
+        <v>0.1414963684510438</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>414.5625</v>
       </c>
     </row>
     <row r="3">
@@ -4328,31 +4328,31 @@
         <v>10</v>
       </c>
       <c r="C3" t="n">
-        <v>666</v>
+        <v>194</v>
       </c>
       <c r="D3" t="n">
-        <v>267</v>
+        <v>95</v>
       </c>
       <c r="E3" t="n">
-        <v>493</v>
+        <v>136</v>
       </c>
       <c r="F3" t="n">
-        <v>320</v>
+        <v>66</v>
       </c>
       <c r="G3" t="n">
-        <v>13.98868884670082</v>
+        <v>4.360094435047358</v>
       </c>
       <c r="H3" t="n">
-        <v>52.53486259514466</v>
+        <v>18.34872942650691</v>
       </c>
       <c r="I3" t="n">
-        <v>0.5419181052129711</v>
+        <v>0.1380650654900817</v>
       </c>
       <c r="J3" t="n">
-        <v>0.9414641577750441</v>
+        <v>0.1610804649535564</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>425.40234375</v>
       </c>
     </row>
     <row r="4">
@@ -4363,31 +4363,31 @@
         <v>5</v>
       </c>
       <c r="C4" t="n">
-        <v>708</v>
+        <v>258</v>
       </c>
       <c r="D4" t="n">
-        <v>283</v>
+        <v>100</v>
       </c>
       <c r="E4" t="n">
-        <v>539</v>
+        <v>198</v>
       </c>
       <c r="F4" t="n">
-        <v>315</v>
+        <v>61</v>
       </c>
       <c r="G4" t="n">
-        <v>16.07347918546293</v>
+        <v>6.659149925690144</v>
       </c>
       <c r="H4" t="n">
-        <v>59.32980544108432</v>
+        <v>27.86360370786861</v>
       </c>
       <c r="I4" t="n">
-        <v>0.4451761174714183</v>
+        <v>0.1702842828817661</v>
       </c>
       <c r="J4" t="n">
-        <v>0.8718546741874879</v>
+        <v>0.4087435747496777</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>425.40234375</v>
       </c>
     </row>
     <row r="5">
@@ -4398,31 +4398,31 @@
         <v>2.5</v>
       </c>
       <c r="C5" t="n">
-        <v>879</v>
+        <v>382</v>
       </c>
       <c r="D5" t="n">
-        <v>270</v>
+        <v>119</v>
       </c>
       <c r="E5" t="n">
-        <v>557</v>
+        <v>247</v>
       </c>
       <c r="F5" t="n">
-        <v>296</v>
+        <v>73</v>
       </c>
       <c r="G5" t="n">
-        <v>49.02228045230731</v>
+        <v>9.385341643821448</v>
       </c>
       <c r="H5" t="n">
-        <v>89.71595810016152</v>
+        <v>37.66826786636375</v>
       </c>
       <c r="I5" t="n">
-        <v>8.099671813426539</v>
+        <v>0.2593262505251905</v>
       </c>
       <c r="J5" t="n">
-        <v>14.20752278342843</v>
+        <v>0.4747780929319549</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>425.40234375</v>
       </c>
     </row>
     <row r="6">
@@ -4433,31 +4433,31 @@
         <v>1.25</v>
       </c>
       <c r="C6" t="n">
-        <v>1332</v>
+        <v>624</v>
       </c>
       <c r="D6" t="n">
-        <v>377</v>
+        <v>189</v>
       </c>
       <c r="E6" t="n">
-        <v>793</v>
+        <v>344</v>
       </c>
       <c r="F6" t="n">
-        <v>395</v>
+        <v>99</v>
       </c>
       <c r="G6" t="n">
-        <v>31.42453185888007</v>
+        <v>14.05331117496826</v>
       </c>
       <c r="H6" t="n">
-        <v>106.0888671710854</v>
+        <v>53.81865542591549</v>
       </c>
       <c r="I6" t="n">
-        <v>1.237932218820784</v>
+        <v>0.3311244177166348</v>
       </c>
       <c r="J6" t="n">
-        <v>3.002654192037877</v>
+        <v>0.6870031729340532</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>425.40234375</v>
       </c>
     </row>
   </sheetData>
@@ -4539,31 +4539,31 @@
         <v>20</v>
       </c>
       <c r="C2" t="n">
-        <v>705</v>
+        <v>135</v>
       </c>
       <c r="D2" t="n">
-        <v>257</v>
+        <v>49</v>
       </c>
       <c r="E2" t="n">
-        <v>497</v>
+        <v>92</v>
       </c>
       <c r="F2" t="n">
-        <v>332</v>
+        <v>36</v>
       </c>
       <c r="G2" t="n">
-        <v>49.61684343672823</v>
+        <v>9.631501971744001</v>
       </c>
       <c r="H2" t="n">
-        <v>178.2478612159612</v>
+        <v>35.28778052190319</v>
       </c>
       <c r="I2" t="n">
-        <v>1.849834322696552</v>
+        <v>0.2344712219201027</v>
       </c>
       <c r="J2" t="n">
-        <v>2.918105075834319</v>
+        <v>0.3917439859360456</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>687.6484375</v>
       </c>
     </row>
     <row r="3">
@@ -4574,31 +4574,31 @@
         <v>10</v>
       </c>
       <c r="C3" t="n">
-        <v>664</v>
+        <v>202</v>
       </c>
       <c r="D3" t="n">
-        <v>207</v>
+        <v>69</v>
       </c>
       <c r="E3" t="n">
-        <v>404</v>
+        <v>136</v>
       </c>
       <c r="F3" t="n">
-        <v>263</v>
+        <v>51</v>
       </c>
       <c r="G3" t="n">
-        <v>45.33196399139706</v>
+        <v>15.23244327539578</v>
       </c>
       <c r="H3" t="n">
-        <v>163.0275517153786</v>
+        <v>55.24015376134776</v>
       </c>
       <c r="I3" t="n">
-        <v>1.280679006013088</v>
+        <v>0.3628585792612282</v>
       </c>
       <c r="J3" t="n">
-        <v>2.023490183171816</v>
+        <v>0.5470570668112484</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>700.08984375</v>
       </c>
     </row>
     <row r="4">
@@ -4609,31 +4609,31 @@
         <v>5</v>
       </c>
       <c r="C4" t="n">
-        <v>711</v>
+        <v>248</v>
       </c>
       <c r="D4" t="n">
-        <v>221</v>
+        <v>94</v>
       </c>
       <c r="E4" t="n">
-        <v>438</v>
+        <v>202</v>
       </c>
       <c r="F4" t="n">
-        <v>240</v>
+        <v>57</v>
       </c>
       <c r="G4" t="n">
-        <v>50.47467044508085</v>
+        <v>23.21078818035312</v>
       </c>
       <c r="H4" t="n">
-        <v>180.8124203648185</v>
+        <v>89.90002425131388</v>
       </c>
       <c r="I4" t="n">
-        <v>1.405742380884475</v>
+        <v>0.7171471484471106</v>
       </c>
       <c r="J4" t="n">
-        <v>2.074586911941878</v>
+        <v>0.8442013307940209</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>702.2421875</v>
       </c>
     </row>
     <row r="5">
@@ -4644,31 +4644,31 @@
         <v>2.5</v>
       </c>
       <c r="C5" t="n">
-        <v>879</v>
+        <v>382</v>
       </c>
       <c r="D5" t="n">
-        <v>285</v>
+        <v>101</v>
       </c>
       <c r="E5" t="n">
-        <v>572</v>
+        <v>220</v>
       </c>
       <c r="F5" t="n">
-        <v>286</v>
+        <v>65</v>
       </c>
       <c r="G5" t="n">
-        <v>61.62499541416764</v>
+        <v>32.78437312971801</v>
       </c>
       <c r="H5" t="n">
-        <v>222.6805510720005</v>
+        <v>120.3712185136974</v>
       </c>
       <c r="I5" t="n">
-        <v>1.673721309634855</v>
+        <v>0.7142942612990724</v>
       </c>
       <c r="J5" t="n">
-        <v>2.512818780844098</v>
+        <v>1.301621933234854</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>705.30859375</v>
       </c>
     </row>
     <row r="6">
@@ -4679,31 +4679,31 @@
         <v>1.25</v>
       </c>
       <c r="C6" t="n">
-        <v>1364</v>
+        <v>626</v>
       </c>
       <c r="D6" t="n">
-        <v>300</v>
+        <v>157</v>
       </c>
       <c r="E6" t="n">
-        <v>720</v>
+        <v>291</v>
       </c>
       <c r="F6" t="n">
-        <v>322</v>
+        <v>57</v>
       </c>
       <c r="G6" t="n">
-        <v>95.48772080696654</v>
+        <v>47.88645441434346</v>
       </c>
       <c r="H6" t="n">
-        <v>324.3207123058382</v>
+        <v>171.6732608885504</v>
       </c>
       <c r="I6" t="n">
-        <v>2.315151128917929</v>
+        <v>1.231310550589112</v>
       </c>
       <c r="J6" t="n">
-        <v>3.523827695287761</v>
+        <v>1.923729777568949</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>705.30859375</v>
       </c>
     </row>
   </sheetData>
@@ -4785,31 +4785,31 @@
         <v>20</v>
       </c>
       <c r="C2" t="n">
-        <v>709</v>
+        <v>138</v>
       </c>
       <c r="D2" t="n">
-        <v>253</v>
+        <v>50</v>
       </c>
       <c r="E2" t="n">
-        <v>506</v>
+        <v>74</v>
       </c>
       <c r="F2" t="n">
-        <v>348</v>
+        <v>36</v>
       </c>
       <c r="G2" t="n">
-        <v>115.8653817678569</v>
+        <v>23.73199123726226</v>
       </c>
       <c r="H2" t="n">
-        <v>405.7470981484512</v>
+        <v>83.02786784479395</v>
       </c>
       <c r="I2" t="n">
-        <v>4.20810675714165</v>
+        <v>0.6523936265148222</v>
       </c>
       <c r="J2" t="n">
-        <v>5.84556619275827</v>
+        <v>1.07542175007984</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>1215.41796875</v>
       </c>
     </row>
     <row r="3">
@@ -4820,31 +4820,31 @@
         <v>10</v>
       </c>
       <c r="C3" t="n">
-        <v>675</v>
+        <v>201</v>
       </c>
       <c r="D3" t="n">
-        <v>213</v>
+        <v>64</v>
       </c>
       <c r="E3" t="n">
-        <v>423</v>
+        <v>123</v>
       </c>
       <c r="F3" t="n">
-        <v>271</v>
+        <v>37</v>
       </c>
       <c r="G3" t="n">
-        <v>111.568812348647</v>
+        <v>37.10530396830291</v>
       </c>
       <c r="H3" t="n">
-        <v>383.76236356562</v>
+        <v>130.0768073198851</v>
       </c>
       <c r="I3" t="n">
-        <v>3.66077060427051</v>
+        <v>1.096488550305366</v>
       </c>
       <c r="J3" t="n">
-        <v>5.478542647440918</v>
+        <v>1.593927752226591</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>1255.41796875</v>
       </c>
     </row>
     <row r="4">
@@ -4855,31 +4855,31 @@
         <v>5</v>
       </c>
       <c r="C4" t="n">
-        <v>720</v>
+        <v>248</v>
       </c>
       <c r="D4" t="n">
-        <v>175</v>
+        <v>73</v>
       </c>
       <c r="E4" t="n">
-        <v>373</v>
+        <v>165</v>
       </c>
       <c r="F4" t="n">
-        <v>209</v>
+        <v>43</v>
       </c>
       <c r="G4" t="n">
-        <v>120.5373222955968</v>
+        <v>56.83620678074658</v>
       </c>
       <c r="H4" t="n">
-        <v>399.3175338545116</v>
+        <v>204.5307487079408</v>
       </c>
       <c r="I4" t="n">
-        <v>3.439200316788628</v>
+        <v>1.766409808304161</v>
       </c>
       <c r="J4" t="n">
-        <v>5.522909677354619</v>
+        <v>2.693274196702987</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>1255.453125</v>
       </c>
     </row>
     <row r="5">
@@ -4890,31 +4890,31 @@
         <v>2.5</v>
       </c>
       <c r="C5" t="n">
-        <v>895</v>
+        <v>394</v>
       </c>
       <c r="D5" t="n">
-        <v>224</v>
+        <v>117</v>
       </c>
       <c r="E5" t="n">
-        <v>456</v>
+        <v>249</v>
       </c>
       <c r="F5" t="n">
-        <v>234</v>
+        <v>65</v>
       </c>
       <c r="G5" t="n">
-        <v>151.8492981974268</v>
+        <v>80.74988319212571</v>
       </c>
       <c r="H5" t="n">
-        <v>506.1342428829521</v>
+        <v>288.3058122112416</v>
       </c>
       <c r="I5" t="n">
-        <v>4.39692868827842</v>
+        <v>2.365673603722825</v>
       </c>
       <c r="J5" t="n">
-        <v>7.157999571063554</v>
+        <v>3.756237500347196</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>1261.7890625</v>
       </c>
     </row>
     <row r="6">
@@ -4925,31 +4925,31 @@
         <v>1.25</v>
       </c>
       <c r="C6" t="n">
-        <v>1379</v>
+        <v>645</v>
       </c>
       <c r="D6" t="n">
-        <v>389</v>
+        <v>146</v>
       </c>
       <c r="E6" t="n">
-        <v>756</v>
+        <v>282</v>
       </c>
       <c r="F6" t="n">
-        <v>335</v>
+        <v>53</v>
       </c>
       <c r="G6" t="n">
-        <v>230.8864183764672</v>
+        <v>125.8319669337943</v>
       </c>
       <c r="H6" t="n">
-        <v>781.3497064244002</v>
+        <v>430.5152797668707</v>
       </c>
       <c r="I6" t="n">
-        <v>6.976126162568104</v>
+        <v>3.153704416472463</v>
       </c>
       <c r="J6" t="n">
-        <v>10.18289490428287</v>
+        <v>5.156607423676176</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>1268.58203125</v>
       </c>
     </row>
   </sheetData>
@@ -4996,10 +4996,10 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0002406371563451914</v>
+        <v>0.000200677477802415</v>
       </c>
       <c r="D2" t="n">
-        <v>0.002128577601215967</v>
+        <v>0.001898559082071692</v>
       </c>
     </row>
     <row r="3">
@@ -5010,10 +5010,10 @@
         <v>0.625</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0002140139010875629</v>
+        <v>0.0001933629787517667</v>
       </c>
       <c r="D3" t="n">
-        <v>0.002857061130385168</v>
+        <v>0.002614993536524815</v>
       </c>
     </row>
     <row r="4">
@@ -5024,10 +5024,10 @@
         <v>0.4166666666666667</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0001470544159514307</v>
+        <v>0.0001380734817467736</v>
       </c>
       <c r="D4" t="n">
-        <v>0.002837705497848469</v>
+        <v>0.002688237124808694</v>
       </c>
     </row>
   </sheetData>
@@ -5074,10 +5074,10 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9306775976600568</v>
+        <v>0.1725371196860733</v>
       </c>
       <c r="D2" t="n">
-        <v>4.639899339378817</v>
+        <v>0.5332765658292701</v>
       </c>
     </row>
     <row r="3">
@@ -5088,10 +5088,10 @@
         <v>0.625</v>
       </c>
       <c r="C3" t="n">
-        <v>0.6803585212136419</v>
+        <v>0.1265220530770271</v>
       </c>
       <c r="D3" t="n">
-        <v>3.227616540063635</v>
+        <v>0.4220446646932949</v>
       </c>
     </row>
     <row r="4">
@@ -5102,10 +5102,10 @@
         <v>0.4166666666666667</v>
       </c>
       <c r="C4" t="n">
-        <v>0.2982555078748266</v>
+        <v>0.05093361677576017</v>
       </c>
       <c r="D4" t="n">
-        <v>2.872413547483303</v>
+        <v>0.3794215006900603</v>
       </c>
     </row>
   </sheetData>
@@ -5152,10 +5152,10 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="C2" t="n">
-        <v>0.3838600042710399</v>
+        <v>0.9311503827811206</v>
       </c>
       <c r="D2" t="n">
-        <v>1.510139840995438</v>
+        <v>3.411682624170548</v>
       </c>
     </row>
     <row r="3">
@@ -5166,10 +5166,10 @@
         <v>0.625</v>
       </c>
       <c r="C3" t="n">
-        <v>0.2731374210944053</v>
+        <v>0.7092897234597401</v>
       </c>
       <c r="D3" t="n">
-        <v>1.106568023438778</v>
+        <v>2.848073779658055</v>
       </c>
     </row>
     <row r="4">
@@ -5180,10 +5180,10 @@
         <v>0.4166666666666667</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1176570706471517</v>
+        <v>0.3062973212630072</v>
       </c>
       <c r="D4" t="n">
-        <v>0.9953817639155014</v>
+        <v>2.586035044363348</v>
       </c>
     </row>
   </sheetData>
@@ -5230,10 +5230,10 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="C2" t="n">
-        <v>0.3283355379509665</v>
+        <v>0.3114835359603785</v>
       </c>
       <c r="D2" t="n">
-        <v>1.039251987149339</v>
+        <v>0.840345297382084</v>
       </c>
     </row>
     <row r="3">
@@ -5244,10 +5244,10 @@
         <v>0.625</v>
       </c>
       <c r="C3" t="n">
-        <v>0.298533192964418</v>
+        <v>0.2760774844604424</v>
       </c>
       <c r="D3" t="n">
-        <v>0.7430302015350815</v>
+        <v>0.6366272297641949</v>
       </c>
     </row>
     <row r="4">
@@ -5258,10 +5258,10 @@
         <v>0.4166666666666667</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1345978273897954</v>
+        <v>0.1206180786920389</v>
       </c>
       <c r="D4" t="n">
-        <v>0.648308009631444</v>
+        <v>0.5490999191424697</v>
       </c>
     </row>
   </sheetData>
@@ -5308,10 +5308,10 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0002335804665463222</v>
+        <v>0.000201023533349233</v>
       </c>
       <c r="D2" t="n">
-        <v>0.002050339435941669</v>
+        <v>0.001901934122173353</v>
       </c>
     </row>
     <row r="3">
@@ -5322,10 +5322,10 @@
         <v>0.625</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0002057849464393328</v>
+        <v>0.0001938748294378169</v>
       </c>
       <c r="D3" t="n">
-        <v>0.002748660703623971</v>
+        <v>0.002621740174625352</v>
       </c>
     </row>
     <row r="4">
@@ -5336,10 +5336,10 @@
         <v>0.4166666666666667</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0001418529383398449</v>
+        <v>0.0001384522444160656</v>
       </c>
       <c r="D4" t="n">
-        <v>0.002741466160015432</v>
+        <v>0.002695839647616204</v>
       </c>
     </row>
   </sheetData>

</xml_diff>